<commit_message>
docs(platform): update org roster, product-side weekly tasklists, backlink disavow baseline, and October MTD 9d tracking
</commit_message>
<xml_diff>
--- a/05_HUBS/financial/financial-hub-roadmap.xlsx
+++ b/05_HUBS/financial/financial-hub-roadmap.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Readme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Performance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Utilities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sitemap" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Banks" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Markets" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="RACI" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Content Plan" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Quick Wins" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utilities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sitemap" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banks" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Markets" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RACI" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Plan" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Wins" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32894,7 +32894,7 @@
       </c>
       <c r="E15" s="87" t="inlineStr">
         <is>
-          <t>Trang overview toàn cảnh thị trường: Bảng tra cứu lãi suất tiền gửi và lãi suất cho vay của 30+ ngân hàng thương mại, lãi suất điều hành NHNN và so sánh biên độ lãi suất thị trường.</t>
+          <t>Trang overview toàn cảnh thị trường: Bảng tra cứu lãi suất tiền gửi và lãi suất cho vay của 40 ngân hàng thương mại, lãi suất điều hành NHNN và so sánh biên độ lãi suất thị trường.</t>
         </is>
       </c>
       <c r="F15" s="88" t="inlineStr">
@@ -33832,7 +33832,7 @@
       </c>
       <c r="C10" s="100" t="inlineStr">
         <is>
-          <t>Bảng Tra Cứu Lãi Suất Ngân Hàng Toàn Cảnh Thị Trường</t>
+          <t>Bảng Tra Cứu Lãi Suất 40 Ngân Hàng Toàn Cảnh Thị Trường</t>
         </is>
       </c>
       <c r="D10" s="101" t="inlineStr">

</xml_diff>

<commit_message>
feat(reports): update MTD performance tracking, task management week 02, news feed, and hub specs
</commit_message>
<xml_diff>
--- a/05_HUBS/financial/financial-hub-roadmap.xlsx
+++ b/05_HUBS/financial/financial-hub-roadmap.xlsx
@@ -32574,7 +32574,7 @@
       </c>
       <c r="E5" s="53" t="inlineStr">
         <is>
-          <t>Cổng trung tâm điều hướng dịch vụ tài chính toàn sàn (5 khối dịch vụ). Đồng thời quy hoạch Cổng Danh Bạ 34 Ngân Hàng kèm 34 Sub-page chi tiết từng ngân hàng trong Sitemap (/tai-chinh/ngan-hang/[bank-slug]).</t>
+          <t>Cổng trung tâm điều hướng dịch vụ tài chính toàn sàn theo 4 trụ cột (Tín Dụng, Tích Lũy, Đầu Tư, Chi Tiêu). Kiến trúc Mega Menu Header mới đang on UAT (khi chuyển sang trang con có menu riêng sẽ tự động co thành Top menu toàn cục). Đồng thời quy hoạch Cổng Danh Bạ 34 Ngân Hàng trong Sitemap.</t>
         </is>
       </c>
       <c r="F5" s="54" t="inlineStr">
@@ -32766,12 +32766,12 @@
       </c>
       <c r="E11" s="66" t="inlineStr">
         <is>
-          <t>Cổng tra cứu tỷ giá và tool quy đổi ngoại tệ (30+ đồng tiền). Đồng thời tạo 8 Sub-page chi tiết theo từng cặp ngoại tệ trong Sitemap (/tai-chinh/ty-gia/[pair-slug]) kèm bảng so sánh đa ngân hàng.</t>
+          <t>Đã Go-live: Cổng tra cứu tỷ giá thị trường và tool quy đổi ngoại tệ (30+ đồng tiền từ 20+ ngân hàng). Đồng thời kết nối hệ thống Sub-page chi tiết theo từng cặp ngoại tệ trong Sitemap.</t>
         </is>
       </c>
       <c r="F11" s="67" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -32798,7 +32798,7 @@
       </c>
       <c r="E12" s="60" t="inlineStr">
         <is>
-          <t>Tạo 8 Sub-page chi tiết theo từng cặp ngoại tệ trong Sitemap (USD/VND, EUR/VND, JPY/VND, CNY/VND, KRW/VND, GBP/VND, AUD/VND, SGD/VND). Mỗi trang tích hợp tool đổi tiền trực tiếp, bảng tỷ giá 20+ bank và biểu đồ 30 ngày.</t>
+          <t>Đang on UAT 5 cặp tiền tệ phổ biến nhất (USD/VND, EUR/VND, JPY/VND, GBP/VND, CNY/VND) kèm tool đổi tiền trực tiếp, bảng tỷ giá đa ngân hàng và biểu đồ biến động; dự kiến Go-live trong tuần này.</t>
         </is>
       </c>
       <c r="F12" s="67" t="inlineStr">
@@ -32830,12 +32830,12 @@
       </c>
       <c r="E13" s="66" t="inlineStr">
         <is>
-          <t>Tool lập ngân sách chi tiêu và chia hũ tiền lương. Nhập thu nhập thực nhận mỗi tháng để tự động chia tiền theo quy tắc 50/30/20 (Thiết yếu 50%, Linh hoạt 30%, Tích lũy 20%) và mô hình 6 Hũ tài chính, kèm cảnh báo bội chi.</t>
+          <t>Đã Go-live: Tool lập ngân sách chi tiêu và chia hũ tiền lương. Nhập thu nhập thực nhận mỗi tháng để tự động chia tiền theo quy tắc 50/30/20 và mô hình 6 Hũ tài chính, kết nối Hũ Chi Tiêu in-app.</t>
         </is>
       </c>
       <c r="F13" s="67" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -32862,7 +32862,7 @@
       </c>
       <c r="E14" s="60" t="inlineStr">
         <is>
-          <t>Cổng gửi tiết kiệm online trên MoMo. Cập nhật biểu lãi suất tiền gửi ưu đãi của các ngân hàng đối tác (Bản Việt, VPBank) với chính sách cộng thêm tới +0.2% lãi suất, kèm công cụ tính tiền lãi theo từng kỳ hạn.</t>
+          <t>Đang review API lãi suất tiền gửi đối tác trên MoMo (Bản Việt, VPBank) với chính sách ưu đãi +0.2% lãi suất, chuẩn bị tích hợp cổng mở sổ online.</t>
         </is>
       </c>
       <c r="F14" s="67" t="inlineStr">
@@ -32894,12 +32894,12 @@
       </c>
       <c r="E15" s="87" t="inlineStr">
         <is>
-          <t>Trang overview toàn cảnh thị trường: Bảng tra cứu lãi suất tiền gửi và lãi suất cho vay của 40 ngân hàng thương mại, lãi suất điều hành NHNN và so sánh biên độ lãi suất thị trường.</t>
+          <t>Đã Go-live: Bảng tra cứu lãi suất 40 ngân hàng toàn cảnh thị trường và công cụ tính lãi gửi tiết kiệm theo số tiền, tự động hiển thị ngân hàng có lãi suất tối ưu nhất.</t>
         </is>
       </c>
       <c r="F15" s="88" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -32926,12 +32926,12 @@
       </c>
       <c r="E16" s="53" t="inlineStr">
         <is>
-          <t>Bảng giá tra cứu chỉ số chứng khoán (/chung-khoan) và bảng tra cứu giá NAV quỹ mở cơ bản quy hoạch under hub (/tai-chinh/chung-chi-quy), phục vụ nhu cầu tích sản dài hạn không tích hợp sàn giao dịch phức tạp.</t>
+          <t>Đang review API dữ liệu giá NAV và tỷ suất sinh lời của quỹ mở (/tai-chinh/chung-chi-quy); chuẩn bị xây dựng bảng giá tra cứu và tool tích sản SIP.</t>
         </is>
       </c>
       <c r="F16" s="69" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In Progress</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(strategy): add SEO/GEO 2027 thesis, update Financial Hub roadmap, October MTD 14d tracking data, and task management
</commit_message>
<xml_diff>
--- a/05_HUBS/financial/financial-hub-roadmap.xlsx
+++ b/05_HUBS/financial/financial-hub-roadmap.xlsx
@@ -12,12 +12,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utilities" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sitemap" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banks" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank Detail Structure" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Markets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RACI" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Plan" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Wins" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank Detail Structure" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Markets" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RACI" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Plan" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Wins" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +32,7 @@
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="56">
+  <fonts count="63">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -349,8 +350,47 @@
       <color rgb="00B45309"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0094A3B8"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="002563EB"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="001E293B"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00276A3C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00334155"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="008C6B00"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="23">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -481,6 +521,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF000000"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF2F8"/>
+        <bgColor rgb="00EDF2F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -639,7 +691,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="159">
+  <cellXfs count="170">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1063,6 +1115,39 @@
     <xf numFmtId="0" fontId="55" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="23" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="24" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1833,6 +1918,509 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="85" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MA TRẬN PHÂN ĐỊNH TRÁCH NHIỆM RACI: WEB PLATFORM x CELL TEAM (FINHUB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>• Web Platform: Xây dựng Sản Phẩm Web (Utilities), Lập Content Plan, Tracking Luồng Web | • FinHub (Cell Team): Tăng Trưởng (Growth), Content QC, Legal QC, Check Luồng In-App</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Hạng Mục / Đầu Việc Triển Khai</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Web Platform Team</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Cell Team (FinHub BU)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Mô Tả Trách Nhiệm Chi Tiết &amp; Tiêu Chí Nghiệm Thu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>NHÓM I: CHIẾN LƯỢC TĂNG TRƯỞNG &amp; VẬN HÀNH SPRINT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>1.1 Quản Trị Mục Tiêu Tăng Trưởng Kinh Doanh (Business Growth &amp; KPIs)</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Co-Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="D5" s="36" t="inlineStr">
+        <is>
+          <t>Cell Team chịu trách nhiệm chính về mục tiêu kinh doanh (Revenue, MAU, Giao dịch tài chính đầu tiên +25% MoM); Web Platform đồng sở hữu và tối ưu hóa phễu Web Traffic (1M MPV, 500K MEU).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>1.2 Lập Kế Hoạch Sprint Web 1 Tháng &amp; Nhịp Check-in 2 Tuần/Lần</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="C6" s="34" t="inlineStr">
+        <is>
+          <t>Co-Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="D6" s="36" t="inlineStr">
+        <is>
+          <t>Web Platform chủ trì tổ chức Sprint Planning đầu tháng để chốt backlog tính năng Web; Cell Team đồng chủ trì check-in ngày 15 &amp; 30 hàng tháng để rà soát tiến độ và xử lý điểm nghẽn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>NHÓM II: XÂY DỰNG SẢN PHẨM WEB &amp; BỘ TIỆN ÍCH (UTILITIES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>2.1 Lập Trình Master Gateway &amp; Giao Diện Cổng Tài Chính (momo.vn/tai-chinh)</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>Consulted (C)</t>
+        </is>
+      </c>
+      <c r="D8" s="36" t="inlineStr">
+        <is>
+          <t>Web Platform chịu trách nhiệm thiết kế UI/UX, lập trình mặt tiền Cổng Khám Phá Tài Chính, Mega Navigation Bar và Dashboard thị trường tổng hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>2.2 Phát Triển Bộ Tiện Ích &amp; Công Cụ Tính Toán Web (Utilities &amp; Calculators)</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>Consulted (C)</t>
+        </is>
+      </c>
+      <c r="D9" s="36" t="inlineStr">
+        <is>
+          <t>Web Platform lập trình các công cụ tiện ích tương tác không cần đăng nhập (Tính Lương, Thuế, Lãi Tiết Kiệm, FIRE Simulator...); Cell Team tư vấn và chuẩn hóa công thức tài chính.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>2.3 Đóng Gói Bộ Công Cụ Tiện Ích Dùng Chung (Embeddable Widgets SDK)</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>Consulted (C)</t>
+        </is>
+      </c>
+      <c r="D10" s="36" t="inlineStr">
+        <is>
+          <t>Web Platform đóng gói các tiện ích thành Web Components nhúng linh hoạt vào các điểm chạm Web MoMo và đối tác ngoài.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>NHÓM III: KẾ HOẠCH NỘI DUNG, KIỂM DUYỆT CHẤT LƯỢNG &amp; PHÁP LÝ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>3.1 Xây Dựng Kế Hoạch Nội Dung &amp; Từ Khóa SEO (Content Plan &amp; MoSpark AI)</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>Consulted (C)</t>
+        </is>
+      </c>
+      <c r="D12" s="36" t="inlineStr">
+        <is>
+          <t>Web Platform chịu trách nhiệm lập kế hoạch nội dung (Content Plan), nghiên cứu từ khóa theo 24 thị trường và vận hành pipeline GenAI trên MoSpark CMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>3.2 Kiểm Duyệt &amp; Đảm Bảo Chất Lượng Nội Dung Tài Chính (Content QC)</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Contributor (R)</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="D13" s="36" t="inlineStr">
+        <is>
+          <t>Cell Team giữ vai trò Key Owner thẩm định và phê duyệt chất lượng chuyên môn (Content QC), đảm bảo tính chuẩn xác của gói tài chính, lãi suất và thuật ngữ nghiệp vụ trước khi xuất bản.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>3.3 Thẩm Định Pháp Lý &amp; Tuân Thủ Quy Định YMYL / NHNN (Legal QC)</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Contributor (R)</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="D14" s="36" t="inlineStr">
+        <is>
+          <t>Cell Team chịu trách nhiệm làm việc với Pháp Chế và đối tác tài chính để kiểm duyệt tính tuân thủ pháp lý (Legal QC), disclaimers và quy định của Ngân hàng Nhà nước.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>NHÓM IV: TRACKING LUỒNG WEB &amp; KIỂM TRA LUỒNG IN-APP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>4.1 Cấu Hình &amp; Tracking Toàn Diện Luồng Web (Web Tracking, GA4, GTM, OneLink, QR)</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>Consulted (C)</t>
+        </is>
+      </c>
+      <c r="D16" s="36" t="inlineStr">
+        <is>
+          <t>Web Platform chịu trách nhiệm toàn bộ hạ tầng đo lường Kênh Web (Web Tracking): GTM, GA4 events, UTM parameters, Appsflyer OneLink và Dynamic Desktop QR Code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>4.2 Kiểm Tra &amp; Tối Ưu Hóa Hành Trình Người Dùng In-App (Check Luồng In-App, Deeplink, eKYC)</t>
+        </is>
+      </c>
+      <c r="B17" s="34" t="inlineStr">
+        <is>
+          <t>Co-Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="D17" s="36" t="inlineStr">
+        <is>
+          <t>Cell Team chịu trách nhiệm kiểm tra và tối ưu hóa luồng In-App (Check Luồng In-App): đảm bảo khi người dùng click CTA Web sẽ mở đúng màn hình App tương ứng, luồng eKYC và kích hoạt giao dịch đầu tiên mượt mà.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>NHÓM V: BÁO CÁO GIẢI TRÌNH &amp; ĐIỀU PHỐI NGUỒN LỰC</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>5.1 Báo Cáo Hiệu Quả Phễu Web-to-App Hàng Tháng Lên Ban Lãnh Đạo IVP</t>
+        </is>
+      </c>
+      <c r="B19" s="34" t="inlineStr">
+        <is>
+          <t>Co-Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="D19" s="36" t="inlineStr">
+        <is>
+          <t>Cell Team chủ trì báo cáo kết quả tăng trưởng kinh doanh; Web Platform đồng chủ trì báo cáo hiệu quả chuyển đổi Kênh Web lên Ban Lãnh Đạo IVP hàng tháng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>5.2 Cơ Chế Rút Lui &amp; Điều Phối Dự Án (Deprioritization Rule)</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Key Owner (A)</t>
+        </is>
+      </c>
+      <c r="C20" s="34" t="inlineStr">
+        <is>
+          <t>Co-Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="D20" s="36" t="inlineStr">
+        <is>
+          <t>Nếu sau 1-2 tháng phối hợp mà Cell Team không tập trung (chậm Content/Legal QC, thiếu deeplink, trễ cam kết), Web Platform sẽ dừng hỗ trợ và chuyển sang làm dự án khác.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="38" t="inlineStr">
+        <is>
+          <t>BẢNG CHÚ GIẢI KÝ HIỆU &amp; NGUYÊN TẮC PHÂN CÔNG TRÁCH NHIỆM:</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>Thuật Ngữ RACI</t>
+        </is>
+      </c>
+      <c r="B23" s="39" t="inlineStr">
+        <is>
+          <t>Tên Tiếng Anh</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>Vai Trò Thực Tế</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>Mô Tả Trách Nhiệm Chi Tiết</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Key Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Accountable &amp; Responsible</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>Chủ Trì &amp; Chịu Trách Nhiệm Chính</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Đội ngũ chịu trách nhiệm giải trình cao nhất (Accountability) trước Ban Lãnh Đạo IVP và trực tiếp thực thi/nghiệm thu hạng mục.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Co-Owner (A/R)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Co-Accountable &amp; Responsible</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Đồng Sở Hữu &amp; Đồng Thực Thi</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Đội ngũ cùng cam kết kết quả đầu ra, chịu trách nhiệm cung cấp chính sách, deeplink, dữ liệu nghiệp vụ và đồng sở hữu KPI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>Contributor (R)</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Responsible Contributor</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Đội Ngũ Thực Thi Hỗ Trợ</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>Đội ngũ trực tiếp tham gia hỗ trợ kỹ thuật, phối hợp thực thi theo đúng cam kết thời hạn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Consulted (C)</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Consulted</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Tham Vấn Chuyên Môn 2 Chiều</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Đội ngũ được tham khảo ý kiến chuyên môn (công thức lãi suất, kiểm duyệt luật tài chính YMYL, góp ý luồng UX) trước khi phát hành.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Informed (I)</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Informed</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Nhận Thông Tin 1 Chiều</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>Đội ngũ nhận báo cáo cập nhật tiến độ định kỳ để nắm bối cảnh liên phòng ban, không bắt buộc tham gia vận hành chi tiết.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A11:D11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6715,7 +7303,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -39924,6 +40512,893 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="68" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="159" t="inlineStr">
+        <is>
+          <t>QUY CHUẨN CẤU TRÚC DỮ LIỆU CÓ CẤU TRÚC (SCHEMA MARKUP &amp; RICH SNIPPETS SPECIFICATION)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="160" t="inlineStr">
+        <is>
+          <t>Đặc tả kỹ thuật các khối Schema JSON-LD độc lập (custom) và chuẩn SEO/GEO cho từng loại trang thuộc Financial Hub, đảm bảo tính mô-đun và không ghi đè schema hiện hữu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="161" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B3" s="161" t="inlineStr">
+        <is>
+          <t>Page Type</t>
+        </is>
+      </c>
+      <c r="C3" s="161" t="inlineStr">
+        <is>
+          <t>Page URL</t>
+        </is>
+      </c>
+      <c r="D3" s="161" t="inlineStr">
+        <is>
+          <t>Schema Script (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="E3" s="161" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F3" s="161" t="inlineStr">
+        <is>
+          <t>Ghi Chú Kỹ Thuật (Technical Notes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="197" customHeight="1">
+      <c r="A4" s="162" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="163" t="inlineStr">
+        <is>
+          <t>Sub-page Cặp Tiền Tệ (Custom Rate)</t>
+        </is>
+      </c>
+      <c r="C4" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/ty-gia/usd-sang-vnd</t>
+        </is>
+      </c>
+      <c r="D4" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "ExchangeRateSpecification",
+  "currency": "USD",
+  "currentExchangeRate": {
+    "@type": "UnitPriceSpecification",
+    "price": 25470,
+    "priceCurrency": "VND",
+    "unitCode": "USD",
+    "unitText": "Đô la Mỹ"
+  }
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Ready to Deploy</t>
+        </is>
+      </c>
+      <c r="F4" s="167" t="inlineStr">
+        <is>
+          <t>Khối Schema ExchangeRateSpecification độc lập 100%, không ghi đè WebApplication và BreadcrumbList có sẵn. Giá niêm yết 25.470 VND dạng số nguyên.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="418" customHeight="1">
+      <c r="A5" s="162" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="163" t="inlineStr">
+        <is>
+          <t>Sub-page Cặp Tiền Tệ (2 Chiều ItemList)</t>
+        </is>
+      </c>
+      <c r="C5" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/ty-gia/usd-sang-vnd#bang-quy-doi</t>
+        </is>
+      </c>
+      <c r="D5" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "ItemList",
+  "name": "Bảng quy đổi tỷ giá USD và VND hôm nay",
+  "itemListElement": [
+    {
+      "@type": "ExchangeRateSpecification",
+      "currency": "USD",
+      "currentExchangeRate": {
+        "@type": "UnitPriceSpecification",
+        "price": 25470,
+        "priceCurrency": "VND",
+        "unitCode": "USD",
+        "unitText": "Đô la Mỹ"
+      }
+    },
+    {
+      "@type": "ExchangeRateSpecification",
+      "currency": "VND",
+      "currentExchangeRate": {
+        "@type": "UnitPriceSpecification",
+        "price": 0.00003926,
+        "priceCurrency": "USD",
+        "unitCode": "VND",
+        "unitText": "Đồng Việt Nam"
+      }
+    }
+  ]
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E5" s="166" t="inlineStr">
+        <is>
+          <t>Ready to Deploy</t>
+        </is>
+      </c>
+      <c r="F5" s="167" t="inlineStr">
+        <is>
+          <t>Tùy chọn mở rộng cho bảng quy đổi 2 chiều: 1 USD = 25.470 VND và 50.000 VND = 1,96 USD (0.00003926).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="197" customHeight="1">
+      <c r="A6" s="162" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="163" t="inlineStr">
+        <is>
+          <t>Sub-page Cặp Tiền Tệ (Programmatic)</t>
+        </is>
+      </c>
+      <c r="C6" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/ty-gia/[pair-slug]</t>
+        </is>
+      </c>
+      <c r="D6" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "ExchangeRateSpecification",
+  "currency": "{CURRENCY_CODE}",
+  "currentExchangeRate": {
+    "@type": "UnitPriceSpecification",
+    "price": {RATE_NUMBER},
+    "priceCurrency": "VND",
+    "unitCode": "{CURRENCY_CODE}",
+    "unitText": "{CURRENCY_NAME}"
+  }
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E6" s="168" t="inlineStr">
+        <is>
+          <t>In Progress (UAT)</t>
+        </is>
+      </c>
+      <c r="F6" s="167" t="inlineStr">
+        <is>
+          <t>Template schema động cho hệ thống sub-pages 8 cặp tiền tệ (EUR, JPY, GBP, KRW, CNY, AUD, SGD). Cắm biến trực tiếp trong component Head.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="197" customHeight="1">
+      <c r="A7" s="162" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="163" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C7" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/lai-suat</t>
+        </is>
+      </c>
+      <c r="D7" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "WebApplication",
+  "name": "Bảng Tra Cứu Lãi Suất 40 Ngân Hàng &amp; Tính Tiền Gửi Tiết Kiệm MoMo",
+  "applicationCategory": "FinanceApplication",
+  "operatingSystem": "Web",
+  "offers": {
+    "@type": "Offer",
+    "price": "0",
+    "priceCurrency": "VND"
+  }
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E7" s="166" t="inlineStr">
+        <is>
+          <t>Done (Go-Live)</t>
+        </is>
+      </c>
+      <c r="F7" s="167" t="inlineStr">
+        <is>
+          <t>Đã Go-Live: Công cụ tính lãi suất tiết kiệm tối ưu theo số tiền và kỳ hạn của 40 ngân hàng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="132" customHeight="1">
+      <c r="A8" s="162" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="163" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C8" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/phan-bo-luong</t>
+        </is>
+      </c>
+      <c r="D8" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "WebApplication",
+  "name": "Công Cụ Phân Bổ Lương 50/30/20 &amp; Mô Hình 6 Hũ Tài Chính MoMo",
+  "applicationCategory": "FinanceApplication",
+  "operatingSystem": "Web"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E8" s="166" t="inlineStr">
+        <is>
+          <t>Done (Go-Live)</t>
+        </is>
+      </c>
+      <c r="F8" s="167" t="inlineStr">
+        <is>
+          <t>Đã Go-Live: Công cụ lập ngân sách thu nhập cá nhân tức thì, điều hướng mở Hũ Chi Tiêu và Túi Thần Tài.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="171" customHeight="1">
+      <c r="A9" s="162" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="163" t="inlineStr">
+        <is>
+          <t>Cổng Danh Mục Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C9" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/ty-gia</t>
+        </is>
+      </c>
+      <c r="D9" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "CurrencyConversionService",
+  "name": "Cổng Tra Cứu Tỷ Giá Ngoại Tệ &amp; Quy Đổi Tiền Tệ MoMo",
+  "description": "Cập nhật tỷ giá 30+ ngoại tệ từ 20+ ngân hàng thương mại Việt Nam",
+  "provider": {
+    "@type": "Organization",
+    "name": "MoMo"
+  }
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E9" s="166" t="inlineStr">
+        <is>
+          <t>Done (Go-Live)</t>
+        </is>
+      </c>
+      <c r="F9" s="167" t="inlineStr">
+        <is>
+          <t>Cổng danh mục tỷ giá thị trường, tích hợp bộ đổi ngoại tệ trực tuyến đa ngân hàng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="132" customHeight="1">
+      <c r="A10" s="162" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="163" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C10" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/tinh-luong</t>
+        </is>
+      </c>
+      <c r="D10" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "WebApplication",
+  "name": "Công Cụ Tính Lương Gross Sang Net 2026 Chuẩn Luật Thuế TNCN",
+  "applicationCategory": "FinanceApplication",
+  "operatingSystem": "Web"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E10" s="166" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F10" s="167" t="inlineStr">
+        <is>
+          <t>Công cụ tự động khấu trừ BHXH 10.5% và biểu thuế lũy tiến 7 bậc mới nhất.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="119" customHeight="1">
+      <c r="A11" s="162" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="163" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C11" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/gia-vang</t>
+        </is>
+      </c>
+      <c r="D11" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "FinancialProduct",
+  "name": "Bảng Tra Cứu Giá Vàng SJC, 9999, DOJI, PNJ Trực Tuyến",
+  "description": "Cập nhật biến động giá vàng mua bán theo thời gian thực"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E11" s="166" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F11" s="167" t="inlineStr">
+        <is>
+          <t>Bảng giá vàng trực tuyến, biểu đồ lịch sử và công cụ quy đổi chỉ/lượng vàng sang tiền mặt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="119" customHeight="1">
+      <c r="A12" s="162" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="163" t="inlineStr">
+        <is>
+          <t>Chuyên Trang Độc Lập (Vertical Hub)</t>
+        </is>
+      </c>
+      <c r="C12" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/diem-tin-dung</t>
+        </is>
+      </c>
+      <c r="D12" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "FinancialService",
+  "name": "Kiểm Tra Điểm Tín Dụng Cá Nhân &amp; Báo Cáo CIC Miễn Phí Trên MoMo",
+  "serviceType": "Credit Scoring"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E12" s="166" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F12" s="167" t="inlineStr">
+        <is>
+          <t>Công cụ giả lập điểm tín dụng cá nhân (150-750), cảnh báo 5 nhóm nợ xấu và thẩm định vay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="119" customHeight="1">
+      <c r="A13" s="162" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="163" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C13" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/gui-tiet-kiem</t>
+        </is>
+      </c>
+      <c r="D13" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "FinancialProduct",
+  "name": "Gửi Tiết Kiệm Online MoMo Hợp Tác Bản Việt &amp; VPBank",
+  "annualPercentageRate": "7.0"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E13" s="168" t="inlineStr">
+        <is>
+          <t>In Progress (Review API)</t>
+        </is>
+      </c>
+      <c r="F13" s="167" t="inlineStr">
+        <is>
+          <t>Đang review API lãi suất tiền gửi đối tác, hưởng ưu đãi cộng thêm 0.2% lãi suất khi mở sổ in-app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="132" customHeight="1">
+      <c r="A14" s="162" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="163" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C14" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/luong-huu</t>
+        </is>
+      </c>
+      <c r="D14" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "WebApplication",
+  "name": "Công Cụ Dự Toán Lương Hưu &amp; Tuổi Nghỉ Hưu Theo Luật Mới",
+  "applicationCategory": "FinanceApplication",
+  "operatingSystem": "Web"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E14" s="166" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F14" s="167" t="inlineStr">
+        <is>
+          <t>Dự toán tuổi nghỉ hưu theo lộ trình và số tiền lương hưu thực nhận tối đa 75% mức lương đóng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="262" customHeight="1">
+      <c r="A15" s="162" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="163" t="inlineStr">
+        <is>
+          <t>Trang Con Chi Tiết (Programmatic Spoke)</t>
+        </is>
+      </c>
+      <c r="C15" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/ngan-hang/[bank-slug]</t>
+        </is>
+      </c>
+      <c r="D15" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "HowTo",
+  "name": "Hướng Dẫn Liên Kết, Nạp Rút Tiền {BANK_NAME} Trên MoMo",
+  "step": [
+    {
+      "@type": "HowToStep",
+      "name": "Liên kết tài khoản",
+      "text": "Vào mục Liên kết ngân hàng, chọn {BANK_NAME} và xác thực thẻ."
+    },
+    {
+      "@type": "HowToStep",
+      "name": "Nạp tiền tức thì",
+      "text": "Chọn nguồn tiền {BANK_NAME}, nhập số tiền và xác nhận miễn phí."
+    }
+  ]
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E15" s="169" t="inlineStr">
+        <is>
+          <t>Planned (Tháng 10)</t>
+        </is>
+      </c>
+      <c r="F15" s="167" t="inlineStr">
+        <is>
+          <t>Cấu trúc 5 khối nội dung cho 34 ngân hàng đối tác, kết hợp HowTo Schema và BankOrCreditUnion Entity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="119" customHeight="1">
+      <c r="A16" s="162" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="163" t="inlineStr">
+        <is>
+          <t>Cổng Danh Mục Master</t>
+        </is>
+      </c>
+      <c r="C16" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/ngan-hang</t>
+        </is>
+      </c>
+      <c r="D16" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "ItemList",
+  "name": "Danh Bạ 34 Ngân Hàng Đối Tác Liên Kết Với MoMo",
+  "numberOfItems": 34
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E16" s="169" t="inlineStr">
+        <is>
+          <t>Planned (Tháng 10)</t>
+        </is>
+      </c>
+      <c r="F16" s="167" t="inlineStr">
+        <is>
+          <t>Danh bạ tổng hợp 34 ngân hàng kết nối, tra cứu hotline CSKH, biểu phí và lãi suất.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="119" customHeight="1">
+      <c r="A17" s="162" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="163" t="inlineStr">
+        <is>
+          <t>Chuyên Trang Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C17" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/chung-chi-quy</t>
+        </is>
+      </c>
+      <c r="D17" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "FinancialProduct",
+  "name": "Bảng Tra Cứu Giá NAV &amp; Tích Sản Chứng Chỉ Quỹ Mở MoMo",
+  "category": "Mutual Fund"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E17" s="168" t="inlineStr">
+        <is>
+          <t>In Progress (Review API)</t>
+        </is>
+      </c>
+      <c r="F17" s="167" t="inlineStr">
+        <is>
+          <t>Đang review API giá NAV từ BU CVS, phục vụ chương trình Thực Tập Sinh Đầu Tư tích sản từ 10.000đ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="119" customHeight="1">
+      <c r="A18" s="162" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="163" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C18" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/tu-do-tai-chinh</t>
+        </is>
+      </c>
+      <c r="D18" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "WebApplication",
+  "name": "Máy Tính Tự Do Tài Chính &amp; Nghỉ Hưu Sớm (FIRE Simulator)",
+  "applicationCategory": "FinanceApplication"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E18" s="169" t="inlineStr">
+        <is>
+          <t>Planned (Tháng 10)</t>
+        </is>
+      </c>
+      <c r="F18" s="167" t="inlineStr">
+        <is>
+          <t>Giả lập thời gian đạt tự do tài chính theo quy tắc 4% an toàn và tích lũy định kỳ SIP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="119" customHeight="1">
+      <c r="A19" s="162" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="163" t="inlineStr">
+        <is>
+          <t>Chuyên Trang Độc Lập (Vertical Hub)</t>
+        </is>
+      </c>
+      <c r="C19" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/chung-khoan</t>
+        </is>
+      </c>
+      <c r="D19" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "FinancialProduct",
+  "name": "Bảng Giá Tra Cứu Chỉ Số Chứng Khoán MoMo CVX",
+  "serviceType": "Securities Brokerage"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E19" s="166" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F19" s="167" t="inlineStr">
+        <is>
+          <t>Chuyên trang chứng khoán liên kết Vietcap CVX, hỗ trợ mở tài khoản và giao dịch từ 1 cổ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="171" customHeight="1">
+      <c r="A20" s="162" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="163" t="inlineStr">
+        <is>
+          <t>Cổng Danh Mục Tiện Ích (Tools Hub)</t>
+        </is>
+      </c>
+      <c r="C20" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/cong-cu</t>
+        </is>
+      </c>
+      <c r="D20" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "CollectionPage",
+  "name": "Tổng Hợp 26 Công Cụ &amp; Tiện Ích Tài Chính Miễn Phí MoMo",
+  "mainEntity": {
+    "@type": "ItemList",
+    "name": "Danh Sách Tiện Ích Financial Hub",
+    "numberOfItems": 26
+  }
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E20" s="169" t="inlineStr">
+        <is>
+          <t>Planned (Tháng 10)</t>
+        </is>
+      </c>
+      <c r="F20" s="167" t="inlineStr">
+        <is>
+          <t>Cổng tập trung toàn bộ 26 tiện ích tài chính (tính lương, lãi suất, tỷ giá, hưu trí, chi phí cột mốc cuộc đời).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="132" customHeight="1">
+      <c r="A21" s="162" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="163" t="inlineStr">
+        <is>
+          <t>Cổng Trung Tâm (Master Hub)</t>
+        </is>
+      </c>
+      <c r="C21" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh</t>
+        </is>
+      </c>
+      <c r="D21" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "FinancialService",
+  "name": "Trung Tâm Tài Chính MoMo (Financial Master Hub)",
+  "url": "https://www.momo.vn/tai-chinh",
+  "serviceType": "Digital Financial Hub"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E21" s="166" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F21" s="167" t="inlineStr">
+        <is>
+          <t>Mặt tiền tổng hợp kết nối 4 trụ cột tài chính toàn website: Tín Dụng, Tích Lũy, Đầu Tư, Chi Tiêu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="119" customHeight="1">
+      <c r="A22" s="162" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="163" t="inlineStr">
+        <is>
+          <t>Trang Danh Mục Blog (Blog Listing)</t>
+        </is>
+      </c>
+      <c r="C22" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/blog</t>
+        </is>
+      </c>
+      <c r="D22" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "Blog",
+  "name": "Cẩm Nang Tài Chính Cá Nhân &amp; Đầu Tư MoMo",
+  "url": "https://www.momo.vn/tai-chinh/blog"
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E22" s="166" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F22" s="167" t="inlineStr">
+        <is>
+          <t>Cổng danh mục bài viết giáo dục tài chính, kiến thức đầu tư và quản lý dòng tiền.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="262" customHeight="1">
+      <c r="A23" s="162" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="163" t="inlineStr">
+        <is>
+          <t>Trang Chi Tiết Bài Viết (Blog Details)</t>
+        </is>
+      </c>
+      <c r="C23" s="164" t="inlineStr">
+        <is>
+          <t>https://www.momo.vn/tai-chinh/blog/[slug]</t>
+        </is>
+      </c>
+      <c r="D23" s="165" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;
+{
+  "@context": "https://schema.org",
+  "@type": "Article",
+  "headline": "{BLOG_TITLE}",
+  "author": {
+    "@type": "Organization",
+    "name": "MoMo"
+  },
+  "publisher": {
+    "@type": "Organization",
+    "name": "MoMo",
+    "logo": {
+      "@type": "ImageObject",
+      "url": "https://homepage.momocdn.net/fileuploads/svg/momo-file-240411162904.svg"
+    }
+  }
+}
+&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="E23" s="166" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="F23" s="167" t="inlineStr">
+        <is>
+          <t>Schema chuẩn Article cho kho 100 bài viết SEO/GEO (50 bài T9 + 50 bài T10).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -41430,7 +42905,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41690,7 +43165,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -42294,507 +43769,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="85" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>MA TRẬN PHÂN ĐỊNH TRÁCH NHIỆM RACI: WEB PLATFORM x CELL TEAM (FINHUB)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="40" t="inlineStr">
-        <is>
-          <t>• Web Platform: Xây dựng Sản Phẩm Web (Utilities), Lập Content Plan, Tracking Luồng Web | • FinHub (Cell Team): Tăng Trưởng (Growth), Content QC, Legal QC, Check Luồng In-App</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Hạng Mục / Đầu Việc Triển Khai</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Web Platform Team</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Cell Team (FinHub BU)</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Mô Tả Trách Nhiệm Chi Tiết &amp; Tiêu Chí Nghiệm Thu</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>NHÓM I: CHIẾN LƯỢC TĂNG TRƯỞNG &amp; VẬN HÀNH SPRINT</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="33" t="inlineStr">
-        <is>
-          <t>1.1 Quản Trị Mục Tiêu Tăng Trưởng Kinh Doanh (Business Growth &amp; KPIs)</t>
-        </is>
-      </c>
-      <c r="B5" s="34" t="inlineStr">
-        <is>
-          <t>Co-Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="D5" s="36" t="inlineStr">
-        <is>
-          <t>Cell Team chịu trách nhiệm chính về mục tiêu kinh doanh (Revenue, MAU, Giao dịch tài chính đầu tiên +25% MoM); Web Platform đồng sở hữu và tối ưu hóa phễu Web Traffic (1M MPV, 500K MEU).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="33" t="inlineStr">
-        <is>
-          <t>1.2 Lập Kế Hoạch Sprint Web 1 Tháng &amp; Nhịp Check-in 2 Tuần/Lần</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="C6" s="34" t="inlineStr">
-        <is>
-          <t>Co-Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="D6" s="36" t="inlineStr">
-        <is>
-          <t>Web Platform chủ trì tổ chức Sprint Planning đầu tháng để chốt backlog tính năng Web; Cell Team đồng chủ trì check-in ngày 15 &amp; 30 hàng tháng để rà soát tiến độ và xử lý điểm nghẽn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>NHÓM II: XÂY DỰNG SẢN PHẨM WEB &amp; BỘ TIỆN ÍCH (UTILITIES)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="33" t="inlineStr">
-        <is>
-          <t>2.1 Lập Trình Master Gateway &amp; Giao Diện Cổng Tài Chính (momo.vn/tai-chinh)</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="C8" s="37" t="inlineStr">
-        <is>
-          <t>Consulted (C)</t>
-        </is>
-      </c>
-      <c r="D8" s="36" t="inlineStr">
-        <is>
-          <t>Web Platform chịu trách nhiệm thiết kế UI/UX, lập trình mặt tiền Cổng Khám Phá Tài Chính, Mega Navigation Bar và Dashboard thị trường tổng hợp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="33" t="inlineStr">
-        <is>
-          <t>2.2 Phát Triển Bộ Tiện Ích &amp; Công Cụ Tính Toán Web (Utilities &amp; Calculators)</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="C9" s="37" t="inlineStr">
-        <is>
-          <t>Consulted (C)</t>
-        </is>
-      </c>
-      <c r="D9" s="36" t="inlineStr">
-        <is>
-          <t>Web Platform lập trình các công cụ tiện ích tương tác không cần đăng nhập (Tính Lương, Thuế, Lãi Tiết Kiệm, FIRE Simulator...); Cell Team tư vấn và chuẩn hóa công thức tài chính.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>2.3 Đóng Gói Bộ Công Cụ Tiện Ích Dùng Chung (Embeddable Widgets SDK)</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="C10" s="37" t="inlineStr">
-        <is>
-          <t>Consulted (C)</t>
-        </is>
-      </c>
-      <c r="D10" s="36" t="inlineStr">
-        <is>
-          <t>Web Platform đóng gói các tiện ích thành Web Components nhúng linh hoạt vào các điểm chạm Web MoMo và đối tác ngoài.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>NHÓM III: KẾ HOẠCH NỘI DUNG, KIỂM DUYỆT CHẤT LƯỢNG &amp; PHÁP LÝ</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>3.1 Xây Dựng Kế Hoạch Nội Dung &amp; Từ Khóa SEO (Content Plan &amp; MoSpark AI)</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="C12" s="37" t="inlineStr">
-        <is>
-          <t>Consulted (C)</t>
-        </is>
-      </c>
-      <c r="D12" s="36" t="inlineStr">
-        <is>
-          <t>Web Platform chịu trách nhiệm lập kế hoạch nội dung (Content Plan), nghiên cứu từ khóa theo 24 thị trường và vận hành pipeline GenAI trên MoSpark CMS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>3.2 Kiểm Duyệt &amp; Đảm Bảo Chất Lượng Nội Dung Tài Chính (Content QC)</t>
-        </is>
-      </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Contributor (R)</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="D13" s="36" t="inlineStr">
-        <is>
-          <t>Cell Team giữ vai trò Key Owner thẩm định và phê duyệt chất lượng chuyên môn (Content QC), đảm bảo tính chuẩn xác của gói tài chính, lãi suất và thuật ngữ nghiệp vụ trước khi xuất bản.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="33" t="inlineStr">
-        <is>
-          <t>3.3 Thẩm Định Pháp Lý &amp; Tuân Thủ Quy Định YMYL / NHNN (Legal QC)</t>
-        </is>
-      </c>
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>Contributor (R)</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="D14" s="36" t="inlineStr">
-        <is>
-          <t>Cell Team chịu trách nhiệm làm việc với Pháp Chế và đối tác tài chính để kiểm duyệt tính tuân thủ pháp lý (Legal QC), disclaimers và quy định của Ngân hàng Nhà nước.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>NHÓM IV: TRACKING LUỒNG WEB &amp; KIỂM TRA LUỒNG IN-APP</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>4.1 Cấu Hình &amp; Tracking Toàn Diện Luồng Web (Web Tracking, GA4, GTM, OneLink, QR)</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="C16" s="37" t="inlineStr">
-        <is>
-          <t>Consulted (C)</t>
-        </is>
-      </c>
-      <c r="D16" s="36" t="inlineStr">
-        <is>
-          <t>Web Platform chịu trách nhiệm toàn bộ hạ tầng đo lường Kênh Web (Web Tracking): GTM, GA4 events, UTM parameters, Appsflyer OneLink và Dynamic Desktop QR Code.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>4.2 Kiểm Tra &amp; Tối Ưu Hóa Hành Trình Người Dùng In-App (Check Luồng In-App, Deeplink, eKYC)</t>
-        </is>
-      </c>
-      <c r="B17" s="34" t="inlineStr">
-        <is>
-          <t>Co-Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="D17" s="36" t="inlineStr">
-        <is>
-          <t>Cell Team chịu trách nhiệm kiểm tra và tối ưu hóa luồng In-App (Check Luồng In-App): đảm bảo khi người dùng click CTA Web sẽ mở đúng màn hình App tương ứng, luồng eKYC và kích hoạt giao dịch đầu tiên mượt mà.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>NHÓM V: BÁO CÁO GIẢI TRÌNH &amp; ĐIỀU PHỐI NGUỒN LỰC</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="33" t="inlineStr">
-        <is>
-          <t>5.1 Báo Cáo Hiệu Quả Phễu Web-to-App Hàng Tháng Lên Ban Lãnh Đạo IVP</t>
-        </is>
-      </c>
-      <c r="B19" s="34" t="inlineStr">
-        <is>
-          <t>Co-Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="D19" s="36" t="inlineStr">
-        <is>
-          <t>Cell Team chủ trì báo cáo kết quả tăng trưởng kinh doanh; Web Platform đồng chủ trì báo cáo hiệu quả chuyển đổi Kênh Web lên Ban Lãnh Đạo IVP hàng tháng.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="33" t="inlineStr">
-        <is>
-          <t>5.2 Cơ Chế Rút Lui &amp; Điều Phối Dự Án (Deprioritization Rule)</t>
-        </is>
-      </c>
-      <c r="B20" s="16" t="inlineStr">
-        <is>
-          <t>Key Owner (A)</t>
-        </is>
-      </c>
-      <c r="C20" s="34" t="inlineStr">
-        <is>
-          <t>Co-Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="D20" s="36" t="inlineStr">
-        <is>
-          <t>Nếu sau 1-2 tháng phối hợp mà Cell Team không tập trung (chậm Content/Legal QC, thiếu deeplink, trễ cam kết), Web Platform sẽ dừng hỗ trợ và chuyển sang làm dự án khác.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="38" t="inlineStr">
-        <is>
-          <t>BẢNG CHÚ GIẢI KÝ HIỆU &amp; NGUYÊN TẮC PHÂN CÔNG TRÁCH NHIỆM:</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="39" t="inlineStr">
-        <is>
-          <t>Thuật Ngữ RACI</t>
-        </is>
-      </c>
-      <c r="B23" s="39" t="inlineStr">
-        <is>
-          <t>Tên Tiếng Anh</t>
-        </is>
-      </c>
-      <c r="C23" s="39" t="inlineStr">
-        <is>
-          <t>Vai Trò Thực Tế</t>
-        </is>
-      </c>
-      <c r="D23" s="39" t="inlineStr">
-        <is>
-          <t>Mô Tả Trách Nhiệm Chi Tiết</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Key Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Accountable &amp; Responsible</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>Chủ Trì &amp; Chịu Trách Nhiệm Chính</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>Đội ngũ chịu trách nhiệm giải trình cao nhất (Accountability) trước Ban Lãnh Đạo IVP và trực tiếp thực thi/nghiệm thu hạng mục.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Co-Owner (A/R)</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Co-Accountable &amp; Responsible</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>Đồng Sở Hữu &amp; Đồng Thực Thi</t>
-        </is>
-      </c>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>Đội ngũ cùng cam kết kết quả đầu ra, chịu trách nhiệm cung cấp chính sách, deeplink, dữ liệu nghiệp vụ và đồng sở hữu KPI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>Contributor (R)</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Responsible Contributor</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>Đội Ngũ Thực Thi Hỗ Trợ</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr">
-        <is>
-          <t>Đội ngũ trực tiếp tham gia hỗ trợ kỹ thuật, phối hợp thực thi theo đúng cam kết thời hạn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Consulted (C)</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Consulted</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>Tham Vấn Chuyên Môn 2 Chiều</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>Đội ngũ được tham khảo ý kiến chuyên môn (công thức lãi suất, kiểm duyệt luật tài chính YMYL, góp ý luồng UX) trước khi phát hành.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Informed (I)</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Informed</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>Nhận Thông Tin 1 Chiều</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>Đội ngũ nhận báo cáo cập nhật tiến độ định kỳ để nắm bối cảnh liên phòng ban, không bắt buộc tham gia vận hành chi tiết.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A11:D11"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(inventory): expand financial keyword inventories, content plans, clustering engine and proposal engine PRD
</commit_message>
<xml_diff>
--- a/05_HUBS/financial/financial-hub-roadmap.xlsx
+++ b/05_HUBS/financial/financial-hub-roadmap.xlsx
@@ -38727,8 +38727,8 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>• Mua sắm &lt; 3tr: 'Đơn hàng [2 triệu] được miễn phí lãi suất hoàn toàn khi thanh toán đúng hạn trong 45 ngày. Kích hoạt Ví Trả Sau để không bị gián đoạn chi tiêu.'
-• Mua sắm &gt; 10tr: 'Đơn hàng [12 triệu] chia nhỏ trả góp chỉ khoảng [1.1 triệu]/tháng. Duy trì lịch sử trả đúng hạn để được tự động nâng hạn mức đến 20 triệu.'</t>
+          <t>• Gentle: 'Chia nhỏ thanh toán thành các kỳ hạn linh hoạt giúp bạn chủ động dòng tiền, giữ lại số tiền nhàn rỗi sinh lời trên Túi Thần Tài.'
+• Roast (Cà Khịa): 'Mê món đồ {item_amount}đ này quá rồi đúng không? Đừng rút hết tiết kiệm mua đứt, chọn trả góp Ví Trả Sau mỗi tháng vài trăm ngàn để ví không bị viêm màng!'</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -38774,8 +38774,8 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>• Khoản vay &lt; 20tr: 'Với khoản vay [15 triệu] trong 12 tháng, mỗi tháng trả khoảng [1.4 triệu]. Hãy đảm bảo số tiền trả góp hàng tháng không vượt quá 30% thu nhập thực nhận.'
-• Cảnh báo lãi vay: 'Để được áp dụng mức lãi suất vay ưu đãi nhất từ đối tác, hãy kiểm tra báo cáo CIC để đảm bảo không có lịch sử nợ quá hạn.'</t>
+          <t>• Gentle: 'Lãi suất tính trên dư nợ giảm dần minh bạch. Mỗi tháng thanh toán {monthly_payment}đ, giải ngân vào Ví MoMo sau 1 phút duyệt.'
+• Roast (Cà Khịa): 'Cần tiền gấp thì vay ngân hàng uy tín trên MoMo, tuyệt đối tránh xa app đen! Trả mỗi tháng cố định {monthly_payment}đ, rõ ràng từng đồng.'</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
@@ -38820,8 +38820,8 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>• Số lượng nhỏ (&lt; 1 chỉ): 'Vàng nhẫn trơn 9999 có biên độ mua - bán hẹp hơn vàng miếng SJC, thích hợp cho tích lũy lâu dài từng chỉ nhỏ. Tích lũy vàng online trên MoMo chỉ từ 0.1 chỉ.'
-• Số tiền lớn (&gt; 1 lượng): 'Vàng đang ở vùng giá biến động mạnh. Hãy cân đối 50% vàng và 50% gửi Tiết Kiệm Online để bảo vệ dòng tiền phòng thủ.'</t>
+          <t>• Gentle: 'Tích lũy từng phân/chỉ vàng là chiến lược bảo toàn sức mua tuyệt vời. Mua Vàng Tài Lộc online trực tiếp trên ứng dụng MoMo.'
+• Roast (Cà Khịa): 'Vàng nhảy múa từng giờ, mua đu đỉnh là tối mất ngủ! Chưa đủ tiền mua nguyên cây thì mua từng phân vàng online trên MoMo, không lo giấu gối sợ trộm.'</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -38867,9 +38867,8 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>• Nhập &lt; 11tr: 'Với mức lương [10 triệu], bạn chưa phải nộp thuế TNCN. Mẹo tích lũy: Trích ngay [1.8 triệu] (20% lương) vào Túi Thần Tài để sau 1 năm có sẵn quỹ dự phòng [22 triệu] sinh lời mỗi ngày.'
-• Nhập 15 - 35tr: 'Với mức lương [30 triệu], bạn chịu khoảng [2.15 triệu] thuế TNCN. Dòng tiền thặng dư sau sinh hoạt khoảng [8-10 triệu]. Mẹo tối ưu: Chia [5 triệu] vào Tiết Kiệm Online và [3 triệu] vào Thực Tập Sinh Đầu Tư.'
-• Nhập &gt; 40tr: 'Với mức lương [60 triệu], thuế TNCN khoảng [9.8 triệu]/tháng. Mẹo quản trị: Đăng ký người phụ thuộc để giảm trừ thuế, đồng thời trích [20 triệu] phân bổ: 50% Tiết Kiệm + 50% Quỹ Cổ Phiếu.'</t>
+          <t>• Gentle: '{net_ratio}% lương Net đã về bản an toàn! Trích ngay 15% cất vào Túi Thần Tài để tiền sinh lời mỗi ngày trước khi tiêu sạch.'
+• Roast (Cà Khịa): ''Bốc hơi' mất {deduction}đ tiền thuế và bảo hiểm nhưng ví vẫn còn {net}đ cầm cự. Trích ngay {save_15}đ vào Hũ trước khi hội săn sale Shopee tìm đến bạn!'</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -38914,8 +38913,8 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>• Rút một lần: 'Rút BHXH một lần sẽ làm mất quyền lợi hưởng lương hưu và BHYT miễn phí trọn đời. Nếu thực sự cần vốn, hãy cân nhắc trích số tiền nhận được gửi Tiết Kiệm Online sinh lời 6.5%/năm.'
-• Khuyến nghị bảo lưu: 'Nếu tiếp tục bảo lưu, bạn sẽ có lương hưu ổn định hàng tháng khi về già. Dùng Túi Thần Tài để giải quyết nhu cầu chi tiêu trước mắt.'</t>
+          <t>• Gentle: 'Rút một lần giải quyết dòng tiền trước mắt ({lump_sum}đ), nhưng bạn mất đi thẻ BHYT trọn đời và lương hưu hàng tháng.'
+• Roast (Cà Khịa): 'Rút một cục {lump_sum}đ tiêu vèo là hết, rồi về già sống bằng tình thương hả bạn ơi? Nếu rút, nhớ trích 40% gửi Tiết Kiệm Online tạo sổ hưu riêng!'</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -38961,8 +38960,8 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>• Độ hụt thu nhập lớn: 'Lương hưu từ BHXH chỉ đáp ứng khoảng [45-60%] chi phí sinh hoạt tuổi già. Mẹo tài chính: Hãy bắt đầu trích [1 triệu]/tháng vào Chứng Chỉ Quỹ SIP từ bây giờ để xây dựng quỹ hưu trí tự thân an nhàn.'
-• Tích lũy sớm: 'Sức mạnh lãi kép trong 20 năm sẽ biến khoản tiết kiệm định kỳ nhỏ thành tài sản lớn. Kết hợp 50% Tiết Kiệm và 50% Quỹ Mở.'</t>
+          <t>• Gentle: 'Lương hưu dự kiến {monthly_pension}đ/tháng có thể chịu áp lực từ lạm phát. Hãy chủ động lập quỹ hưu trí bổ sung ngay từ hôm nay.'
+• Roast (Cà Khịa): 'Nghỉ hưu với {monthly_pension}đ sau 20 năm nữa chỉ đủ ăn bánh mì uống nước lọc. Tích sản SIP từ 10.000đ/ngày để khi về già thảnh thơi đi du lịch!'</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -39008,8 +39007,8 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>• Nợ Nhóm 1 (Chuẩn): 'Điểm tín dụng của bạn đang ở mức tốt. Duy trì không dùng quá 70% hạn mức thẻ để được ưu tiên nâng hạn mức vay tiêu dùng in-app.'
-• Nợ Nhóm 2 (Cần chú ý): 'Khoản trễ hạn khiến hồ sơ rơi vào Nhóm 2. Hãy tất toán ngay dư nợ trong 3 ngày tới để ngăn chặn hồ sơ chuyển sang nợ xấu Nhóm 3 trên hệ thống CIC Quốc Gia.'</t>
+          <t>• Gentle: 'Điểm tín dụng của bạn thuộc nhóm Ưu tú ({credit_score} điểm), đủ điều kiện mở hạn mức tài chính cao nhất trên MoMo.'
+• Roast (Cà Khịa): 'Uy tín ngời ngời, hồ sơ sạch tinh tươm! Điểm đẹp thế này mà không mở Ví Trả Sau hạn mức tới 20 triệu nhận 45 ngày miễn lãi thì quá phí.'</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -39054,8 +39053,8 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>• Đổi tiền du lịch / công tác: 'Tỷ giá ngoại tệ biến động liên tục. Chuyển đổi dòng tiền sang VND gửi Tiết Kiệm Online MoMo nhận lãi suất lên tới 6.5%/năm cao hơn giữ ngoại tệ.'
-• Đầu tư ngoại tệ: 'Đa dạng hóa danh mục tài sản bằng cách kết hợp gửi Tiết kiệm và tham gia Thực Tập Sinh Đầu Tư.'</t>
+          <t>• Gentle: 'Theo dõi sát biểu đồ biến động để chọn thời điểm đổi tiền tối ưu. Khi đi du lịch, quét mã QR thanh toán quốc tế trực tiếp qua MoMo.'
+• Roast (Cà Khịa): 'Tính đổi tiền đi vi vu nước ngoài hả bạn ơi? Đổi tiền mặt cồng kềnh dễ rơi mất, dùng MoMo quét mã QR thanh toán quốc tế không tốn phí chuyển đổi!'</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -39101,8 +39100,8 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>• Chi phí thiết yếu &gt; 65%: 'Chi phí cố định đang chiếm [68%] thu nhập, vượt ngưỡng an toàn 50%. Hãy dùng Hũ Chi Tiêu MoMo để kiểm soát chặt chẽ ngân sách sinh hoạt.'
-• Tích lũy đạt &gt;= 20%: 'Bạn đang trích được [4 triệu] (20% thu nhập) để tích sản. Gợi ý: Tự động hóa việc trích tiền vào Tiết Kiệm TKO và Quỹ Mở SIP ngay ngày nhận lương.'</t>
+          <t>• Gentle: 'Khoản chi tiêu sở thích đang chiếm {want_ratio}% thu nhập. Cài đặt hạn mức Hũ Chi Tiêu tuần để bảo vệ quỹ tiết kiệm tương lai.'
+• Roast (Cà Khịa): 'Nghe nói bạn định tiết kiệm, nhưng giỏ hàng Shopee và ly trà sữa size L đã nói 'không'. Khóa trần hạn mức bằng Hũ Chi Tiêu trước khi ăn mì tôm ngày 20!'</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -39148,8 +39147,8 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>• Số tiền &lt; 20tr, kỳ hạn ngắn: 'Với số tiền [10 triệu] gửi ngắn hạn, tiền lãi ngân hàng chênh lệch không đáng kể. Hãy để trong Túi Thần Tài nhận lời mỗi ngày và rút ra chi tiêu bất kỳ lúc nào không lo mất lãi.'
-• Số tiền &gt; 100tr, kỳ hạn 12 tháng: 'Với số tiền [300 triệu], chênh lệch 0.5% lãi suất mang lại thêm [1.5 triệu] tiền lời mỗi năm. Mở sổ Tiết kiệm Bản Việt trên MoMo hiện được cộng thêm 0.2% lãi suất ưu đãi.'</t>
+          <t>• Gentle: 'Gửi tại {selected_bank} bạn nhận {user_interest}đ. Gửi qua đối tác Bản Việt/VPBank trên MoMo, nhận thêm chênh lệch {gap_interest}đ tiền lãi.'
+• Roast (Cà Khịa): 'Cùng là số tiền này mà gửi ở đây bạn đang 'tặng không' cho ngân hàng {gap_interest}đ tiền lãi. Mở sổ trên MoMo nhận thêm +0.2% lãi suất, đủ uống trà sữa cả năm!'</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -39194,7 +39193,8 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>• Tuổi trẻ (&lt; 30 tuổi): 'Bạn có lợi thế lớn về thời gian. Chỉ cần trích [1.5 triệu]/tháng đầu tư Chứng Chỉ Quỹ SIP với lợi suất kỳ vọng 12%/năm, sức mạnh lãi kép sau 15 năm sẽ mang lại hơn [750 triệu] đồng.'</t>
+          <t>• Gentle: 'Để nghỉ hưu ở tuổi {retire_age}, bạn cần khối tài sản sinh lời ròng {target_asset}đ theo quy tắc 4% an toàn. Bắt đầu tích sản định kỳ quỹ mở ngay hôm nay.'
+• Roast (Cà Khịa): 'Muốn 35 tuổi đã thảnh thơi đi câu cá ngắm hoàng hôn? Với tốc độ tiêu tiền hiện tại thì 65 tuổi bạn vẫn đang cày deadline đấy! Bắt tay vào tích sản SIP ngay!'</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -39286,8 +39286,8 @@
       </c>
       <c r="E16" s="155" t="inlineStr">
         <is>
-          <t>• Chi phí &gt; 150tr: "Bạn cần đặt cọc trước khoảng [60 triệu] trước ngày cưới. Sử dụng Ví Trả Sau hoặc Vay Nhanh MoMo để thanh toán cọc nhà hàng và tất toán ngay sau tiệc cưới từ tiền mừng."
-• Kế hoạch sớm: "Hãy tạo Hũ Cưới Hỏi để tích lũy trước 6-12 tháng."</t>
+          <t>• Gentle: 'Chi phí tiệc cưới đang chênh lệch cao so với dự phòng. Hãy cân nhắc tối ưu các khoản decor hoặc kích hoạt nguồn vốn đòn bẩy ngắn hạn an toàn.'
+• Roast (Cà Khịa): 'Tính toán cho thấy đám cưới cần tối thiểu 35 mâm cỗ để hòa vốn. Nếu hội bạn thân đi phong bì 300k thì cô dâu chú rể chuẩn bị rửa bát trừ nợ! Bật Ví Trả Sau dự phòng 20 triệu ngay!'</t>
         </is>
       </c>
       <c r="F16" s="155" t="inlineStr">
@@ -39380,8 +39380,8 @@
       </c>
       <c r="E18" s="155" t="inlineStr">
         <is>
-          <t>• Chi phí tháng đầu quá cao: "Tháng đầu ra riêng bạn cần chuẩn bị khoảng [15 triệu] (gồm cọc và sắm đồ). Dùng Ví Trả Sau để chia nhỏ trả góp đồ gia dụng, tránh làm cạn kiệt tiền mặt phòng thân."
-• Cảnh báo: "Tiền thuê nhà đang chiếm [38%] lương, hãy cân nhắc tìm bạn ở ghép."</t>
+          <t>• Gentle: 'Chi phí nhà ở vượt quá ngưỡng an toàn tài chính (30%). Nên tìm bạn ở ghép hoặc lựa chọn khu vực có chi phí tối ưu hơn.'
+• Roast (Cà Khịa): 'Căn phòng có ban công chill thật đấy, nhưng tiền thuê ngốn gần nửa tháng lương thì tối về chỉ có nước ngắm trăng uống nước lọc. Đi làm cả tháng chỉ để nuôi chủ nhà thôi bạn ơi!'</t>
         </is>
       </c>
       <c r="F18" s="155" t="inlineStr">
@@ -39474,8 +39474,8 @@
       </c>
       <c r="E20" s="155" t="inlineStr">
         <is>
-          <t>• Sức mạnh tích sản nhỏ: "Chỉ với [20.000đ/ngày] (bằng 1 cốc cà phê), sau 5 năm bạn tích lũy được [52 triệu đồng], trong đó tiền lời từ lãi kép đạt hơn [16 triệu]. Bắt đầu ngay với gói Thực Tập Sinh Đầu Tư trên MoMo."
-• Thời gian dài (&gt; 10 năm): "Sức mạnh lãi kép sẽ giúp tài sản của bạn tăng gấp 3 lần số vốn bỏ ra."</t>
+          <t>• Gentle: 'Tích lũy đều đặn 10.000đ/ngày mang lại sức mạnh lãi kép vượt trội. Thích hợp cho mục tiêu tích sản tài sản tăng trưởng trung và dài hạn.'
+• Roast (Cà Khịa): '10.000đ mỗi ngày không làm bạn nghèo đi, nhưng bỏ qua lãi kép 12%/năm thì 5 năm nữa nhìn lại bạn bè mua nhà còn mình vẫn mua ly trà sữa!'</t>
         </is>
       </c>
       <c r="F20" s="155" t="inlineStr">

</xml_diff>

<commit_message>
feat: optimize url project resolver, sync performance metrics, and add gsc zero impression analysis
</commit_message>
<xml_diff>
--- a/05_HUBS/financial/financial-hub-roadmap.xlsx
+++ b/05_HUBS/financial/financial-hub-roadmap.xlsx
@@ -32,7 +32,7 @@
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="63">
+  <fonts count="65">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -389,8 +389,18 @@
       <color rgb="001E3A8A"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001F4E78"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00047857"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
-  <fills count="25">
+  <fills count="26">
     <fill>
       <patternFill/>
     </fill>
@@ -533,6 +543,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00EDF2F8"/>
         <bgColor rgb="00EDF2F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -691,7 +707,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="170">
+  <cellXfs count="189">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1148,6 +1164,61 @@
     <xf numFmtId="0" fontId="62" fillId="24" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -38056,7 +38127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -38194,7 +38265,7 @@
       </c>
       <c r="E5" s="53" t="inlineStr">
         <is>
-          <t>Cổng trung tâm điều hướng dịch vụ tài chính toàn sàn theo 4 trụ cột (Tín Dụng, Tích Lũy, Đầu Tư, Chi Tiêu). Kiến trúc Mega Menu Header mới đang on UAT (khi chuyển sang trang con có menu riêng sẽ tự động co thành Top menu toàn cục). Đồng thời quy hoạch Cổng Danh Bạ 34 Ngân Hàng trong Sitemap.</t>
+          <t>Cổng trung tâm điều hướng dịch vụ tài chính Kênh Web theo 4 trụ cột (Tín Dụng, Tích Lũy, Đầu Tư, Chi Tiêu). Kiến trúc Mega Menu Header mới đang on UAT (khi chuyển sang trang con có menu riêng sẽ tự động co thành Top menu toàn cục). Đồng thời quy hoạch Cổng Danh Bạ 34 Ngân Hàng trong Sitemap.</t>
         </is>
       </c>
       <c r="F5" s="54" t="inlineStr">
@@ -38322,7 +38393,7 @@
       </c>
       <c r="E9" s="53" t="inlineStr">
         <is>
-          <t>Tool tính tiền rút BHXH một lần. Nhập số năm đóng và mức lương bình quân đóng bảo hiểm để ước tính tổng số tiền trợ cấp một lần được nhận theo quy định mới nhất của Luật BHXH.</t>
+          <t>Tool tính tiền rút BHXH một lần. Nhập số năm đóng và mức lương bình quân đóng bảo hiểm để ước tính tổng tiền trợ cấp (tích hợp trực tiếp vào /tai-chinh/luong-huu, không tạo URL bảo hiểm riêng biệt).</t>
         </is>
       </c>
       <c r="F9" s="54" t="inlineStr">
@@ -38524,102 +38595,165 @@
       </c>
     </row>
     <row r="16" ht="54" customHeight="1">
-      <c r="A16" s="49" t="inlineStr">
+      <c r="A16" s="170" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B16" s="50" t="inlineStr">
+      <c r="B16" s="171" t="inlineStr">
         <is>
           <t>Tháng 10/2026</t>
         </is>
       </c>
-      <c r="C16" s="51" t="inlineStr">
-        <is>
-          <t>Đầu Tư &amp; Chứng Chỉ Quỹ</t>
-        </is>
-      </c>
-      <c r="D16" s="52" t="inlineStr">
-        <is>
-          <t>Chứng Khoán &amp; Chứng Chỉ Quỹ</t>
-        </is>
-      </c>
-      <c r="E16" s="53" t="inlineStr">
-        <is>
-          <t>Đang review API dữ liệu giá NAV và tỷ suất sinh lời của quỹ mở (/tai-chinh/chung-chi-quy); chuẩn bị xây dựng bảng giá tra cứu và tool tích sản SIP.</t>
-        </is>
-      </c>
-      <c r="F16" s="69" t="inlineStr">
+      <c r="C16" s="172" t="inlineStr">
+        <is>
+          <t>Đầu Tư &amp; Tích Sản</t>
+        </is>
+      </c>
+      <c r="D16" s="173" t="inlineStr">
+        <is>
+          <t>Cổng Chứng Khoán Master &amp; 30 Dynamic Profiles VN30</t>
+        </is>
+      </c>
+      <c r="E16" s="174" t="inlineStr">
+        <is>
+          <t>Xây dựng Cổng Master /tai-chinh/chung-khoan và 30 trang Dynamic Ticker Profile cho toàn bộ rổ VN30 (/tai-chinh/chung-khoan/[ticker]) trong Sitemap. Tích hợp máy tính Stock DCA Backtester và Thước đo Sức khỏe MoMo Stock Health Score 1-100, phục vụ chiến lược tích sản cổ phiếu lô lẻ từ 10.000đ kết nối đối tác CVS.</t>
+        </is>
+      </c>
+      <c r="F16" s="175" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
     </row>
     <row r="17" ht="54" customHeight="1">
-      <c r="A17" s="56" t="inlineStr">
+      <c r="A17" s="176" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B17" s="57" t="inlineStr">
+      <c r="B17" s="177" t="inlineStr">
         <is>
           <t>Tháng 10/2026</t>
         </is>
       </c>
-      <c r="C17" s="58" t="inlineStr">
+      <c r="C17" s="178" t="inlineStr">
+        <is>
+          <t>Đầu Tư &amp; Tích Sản</t>
+        </is>
+      </c>
+      <c r="D17" s="179" t="inlineStr">
+        <is>
+          <t>Chứng Chỉ Quỹ &amp; Máy Tính Tích Sản SIP</t>
+        </is>
+      </c>
+      <c r="E17" s="180" t="inlineStr">
+        <is>
+          <t>Đang review API dữ liệu giá NAV và tỷ suất sinh lời của 30 quỹ mở từ BU CVS; xây dựng Cổng /tai-chinh/chung-chi-quy và 30 trang chi tiết quỹ (/tai-chinh/chung-chi-quy/[fund-slug]) trong Sitemap kèm máy tính tích sản SIP từ 10.000đ/ngày. Tích hợp cơ chế Dual-conversion chuyển đổi chéo trực tiếp từ các trang mã cổ phiếu.</t>
+        </is>
+      </c>
+      <c r="F17" s="175" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1">
+      <c r="A18" s="170" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="B18" s="171" t="inlineStr">
+        <is>
+          <t>Tháng 10/2026</t>
+        </is>
+      </c>
+      <c r="C18" s="172" t="inlineStr">
+        <is>
+          <t>Kiến Trúc &amp; Tái Định Tuyến URL</t>
+        </is>
+      </c>
+      <c r="D18" s="173" t="inlineStr">
+        <is>
+          <t>Di Chuyển &amp; 301 Redirect 7 Trang Standalone Về /tai-chinh/*</t>
+        </is>
+      </c>
+      <c r="E18" s="174" t="inlineStr">
+        <is>
+          <t>Thực hiện 301 Redirect tại Edge CDN cho 7 trang standalone về /tai-chinh/* (/nhan-tien-quoc-te, /quy-nhom, /thanh-toan-the-tin-dung, /quan-ly-chi-tieu, /chung-khoan, /chung-chi-quy, /tui-sinh-loi). Cam kết bảo toàn: Ví Trả Sau (/vi-tra-sau), Vay Nhanh (/vay-nhanh), Điểm Tín Dụng (/diem-tin-dung) tuyệt đối giữ nguyên URL root độc lập, không đưa về under /tai-chinh/*. Loại trừ hoàn toàn nhóm Bảo hiểm khỏi Financial Hub.</t>
+        </is>
+      </c>
+      <c r="F18" s="175" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1">
+      <c r="A19" s="176" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="B19" s="177" t="inlineStr">
+        <is>
+          <t>Tháng 10/2026</t>
+        </is>
+      </c>
+      <c r="C19" s="178" t="inlineStr">
         <is>
           <t>Dòng Tiền &amp; Tiêu Dùng</t>
         </is>
       </c>
-      <c r="D17" s="59" t="inlineStr">
+      <c r="D19" s="179" t="inlineStr">
         <is>
           <t>Quản Lý Dòng Tiền &amp; Tiêu Dùng</t>
         </is>
       </c>
-      <c r="E17" s="60" t="inlineStr">
-        <is>
-          <t>Tool tính dòng tiền tự do và quỹ khẩn cấp. Nhập tổng thu nhập và các khoản chi cố định hàng tháng để tính số tiền thặng dư tự do (Free Cash Flow), quy mô quỹ dự phòng rủi ro cần có (3 - 6 tháng chi phí) và số tháng tài chính cầm cự nếu mất nguồn thu.</t>
-        </is>
-      </c>
-      <c r="F17" s="69" t="inlineStr">
+      <c r="E19" s="180" t="inlineStr">
+        <is>
+          <t>Tool tính dòng tiền tự do và quỹ khẩn cấp. Nhập tổng thu nhập và các khoản chi cố định hàng tháng để tính số tiền thặng dư tự do (Free Cash Flow), quy mô quỹ dự phòng rủi ro cần có (3 - 6 tháng chi phí) và số tháng tài chính cầm cự nếu mất nguồn thu. Định tuyến trang /tai-chinh/dong-tien trong Sitemap.</t>
+        </is>
+      </c>
+      <c r="F19" s="181" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="54" customHeight="1">
-      <c r="A18" s="92" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="170" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B18" s="93" t="inlineStr">
+      <c r="B20" s="171" t="inlineStr">
         <is>
           <t>Tháng 10/2026</t>
         </is>
       </c>
-      <c r="C18" s="94" t="inlineStr">
+      <c r="C20" s="172" t="inlineStr">
         <is>
           <t>Tích Sản &amp; Hưu Trí</t>
         </is>
       </c>
-      <c r="D18" s="95" t="inlineStr">
+      <c r="D20" s="173" t="inlineStr">
         <is>
           <t>Đầu Tư &amp; Tích Sản FIRE</t>
         </is>
       </c>
-      <c r="E18" s="96" t="inlineStr">
+      <c r="E20" s="174" t="inlineStr">
         <is>
           <t>Tool lập kế hoạch tự do tài chính và nghỉ hưu sớm. Tạo trang độc lập /tai-chinh/tu-do-tai-chinh trong Sitemap theo quy tắc rút 4% an toàn và lộ trình tích sản hàng tháng.</t>
         </is>
       </c>
-      <c r="F18" s="97" t="inlineStr">
+      <c r="F20" s="181" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="54" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -39346,7 +39480,7 @@
       </c>
       <c r="G17" s="156" t="inlineStr">
         <is>
-          <t>Thực Tập Sinh Đầu Tư, Tiết Kiệm, Bảo Hiểm</t>
+          <t>Thực Tập Sinh Đầu Tư, Tiết Kiệm, Hũ Tài Chính</t>
         </is>
       </c>
       <c r="H17" s="157" t="inlineStr">
@@ -39932,13 +40066,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="68" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -39951,7 +40085,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="32" t="inlineStr">
         <is>
-          <t>Bản đồ định tuyến toàn bộ 26 trang thuộc Financial Hub gồm: Cổng trung tâm, Cổng tiện ích /tai-chinh/cong-cu, các Tool cấp 1 trực thuộc /tai-chinh/*, hệ thống Sub-page 8 cặp ngoại tệ, chuyên trang độc lập và blog hub.</t>
+          <t>Bản đồ định tuyến toàn bộ hệ thống URLs thuộc Financial Hub (loại trừ hoàn toàn nhóm Bảo hiểm thuộc Insurtech Hub). Ví Trả Sau (/vi-tra-sau), Vay Nhanh (/vay-nhanh), Điểm Tín Dụng (/diem-tin-dung) giữ nguyên URL root độc lập, tuyệt đối không đưa về under /tai-chinh/*. Toàn bộ các trang tài chính chuyển về /tai-chinh/* được liệt kê chi tiết dưới đây.</t>
         </is>
       </c>
     </row>
@@ -39978,522 +40112,2282 @@
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="98" t="n">
+      <c r="A4" s="182" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="99" t="inlineStr">
+      <c r="B4" s="183" t="inlineStr">
         <is>
           <t>Cổng Trung Tâm (Master Hub)</t>
         </is>
       </c>
-      <c r="C4" s="100" t="inlineStr">
+      <c r="C4" s="178" t="inlineStr">
         <is>
           <t>Financial Master Hub MoMo</t>
         </is>
       </c>
-      <c r="D4" s="101" t="inlineStr">
+      <c r="D4" s="184" t="inlineStr">
         <is>
           <t>/tai-chinh</t>
         </is>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="98" t="n">
+      <c r="A5" s="185" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="99" t="inlineStr">
+      <c r="B5" s="186" t="inlineStr">
         <is>
           <t>Cổng Danh Mục Tiện Ích (Tools Hub)</t>
         </is>
       </c>
-      <c r="C5" s="100" t="inlineStr">
+      <c r="C5" s="172" t="inlineStr">
         <is>
           <t>Tổng Hợp Công Cụ &amp; Tiện Ích Tài Chính MoMo</t>
         </is>
       </c>
-      <c r="D5" s="101" t="inlineStr">
+      <c r="D5" s="187" t="inlineStr">
         <is>
           <t>/tai-chinh/cong-cu</t>
         </is>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="98" t="n">
+      <c r="A6" s="182" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="99" t="inlineStr">
-        <is>
-          <t>Chuyên Trang Độc Lập (Vertical Hub)</t>
-        </is>
-      </c>
-      <c r="C6" s="100" t="inlineStr">
-        <is>
-          <t>Điểm Tín Dụng &amp; Tra Cứu CIC</t>
-        </is>
-      </c>
-      <c r="D6" s="101" t="inlineStr">
+      <c r="B6" s="183" t="inlineStr">
+        <is>
+          <t>Trang Độc Lập Root (Không Đổi URL)</t>
+        </is>
+      </c>
+      <c r="C6" s="178" t="inlineStr">
+        <is>
+          <t>Điểm Tín Dụng &amp; Tra Cứu CIC (Root URL)</t>
+        </is>
+      </c>
+      <c r="D6" s="184" t="inlineStr">
         <is>
           <t>/diem-tin-dung</t>
         </is>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="98" t="n">
+      <c r="A7" s="185" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="99" t="inlineStr">
+      <c r="B7" s="186" t="inlineStr">
+        <is>
+          <t>Trang Độc Lập Root (Không Đổi URL)</t>
+        </is>
+      </c>
+      <c r="C7" s="172" t="inlineStr">
+        <is>
+          <t>Vay Tiêu Dùng Nhanh Trực Tuyến (Root URL)</t>
+        </is>
+      </c>
+      <c r="D7" s="187" t="inlineStr">
+        <is>
+          <t>/vay-nhanh</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="182" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="183" t="inlineStr">
+        <is>
+          <t>Trang Độc Lập Root (Không Đổi URL)</t>
+        </is>
+      </c>
+      <c r="C8" s="178" t="inlineStr">
+        <is>
+          <t>Ví Trả Sau MoMo &amp; Mua Sắm Trả Góp 0% (Root URL)</t>
+        </is>
+      </c>
+      <c r="D8" s="184" t="inlineStr">
+        <is>
+          <t>/vi-tra-sau</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="185" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="186" t="inlineStr">
+        <is>
+          <t>Trang Độc Lập Root (Không Đổi URL)</t>
+        </is>
+      </c>
+      <c r="C9" s="172" t="inlineStr">
+        <is>
+          <t>Thẻ Tín Dụng Quốc Tế Hoàn Tiền (Root URL)</t>
+        </is>
+      </c>
+      <c r="D9" s="187" t="inlineStr">
+        <is>
+          <t>/the-tin-dung</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="182" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="183" t="inlineStr">
+        <is>
+          <t>Trang Dịch Vụ Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C10" s="178" t="inlineStr">
+        <is>
+          <t>Cổng Master Chứng Khoán &amp; Tích Sản Cổ Phiếu Lô Lẻ Từ 10.000đ</t>
+        </is>
+      </c>
+      <c r="D10" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="185" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="186" t="inlineStr">
+        <is>
+          <t>Trang Dịch Vụ Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C11" s="172" t="inlineStr">
+        <is>
+          <t>Cổng Tra Cứu Giá NAV &amp; Tích Sản Quỹ Mở MoMo</t>
+        </is>
+      </c>
+      <c r="D11" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="182" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="183" t="inlineStr">
+        <is>
+          <t>Trang Dịch Vụ Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C12" s="178" t="inlineStr">
+        <is>
+          <t>Túi Sinh Lời (Túi Thần Tài) - Tích Lũy Sinh Lời Mỗi Ngày</t>
+        </is>
+      </c>
+      <c r="D12" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/tui-sinh-loi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="185" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="186" t="inlineStr">
+        <is>
+          <t>Trang Dịch Vụ Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C13" s="172" t="inlineStr">
+        <is>
+          <t>Cổng Chuyển Tiền &amp; Nhận Tiền Quốc Tế MoMo</t>
+        </is>
+      </c>
+      <c r="D13" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/nhan-tien-quoc-te</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="182" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="183" t="inlineStr">
+        <is>
+          <t>Trang Dịch Vụ Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C14" s="178" t="inlineStr">
+        <is>
+          <t>Quỹ Nhóm &amp; Quản Lý Quỹ Chung MoMo</t>
+        </is>
+      </c>
+      <c r="D14" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/quy-nhom</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="185" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="186" t="inlineStr">
+        <is>
+          <t>Trang Dịch Vụ Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C15" s="172" t="inlineStr">
+        <is>
+          <t>Thanh Toán Dư Nợ Thẻ Tín Dụng Đa Ngân Hàng</t>
+        </is>
+      </c>
+      <c r="D15" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/thanh-toan-the-tin-dung</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="182" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="183" t="inlineStr">
+        <is>
+          <t>Trang Dịch Vụ Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C16" s="178" t="inlineStr">
+        <is>
+          <t>Cổng Quản Lý Chi Tiêu Cá Nhân MoMo</t>
+        </is>
+      </c>
+      <c r="D16" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/quan-ly-chi-tieu</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="185" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="186" t="inlineStr">
         <is>
           <t>Công Cụ Tiện Ích Under /tai-chinh</t>
         </is>
       </c>
-      <c r="C7" s="100" t="inlineStr">
-        <is>
-          <t>Bảng Giá Vàng SJC, 9999 Mới Nhất</t>
-        </is>
-      </c>
-      <c r="D7" s="101" t="inlineStr">
+      <c r="C17" s="172" t="inlineStr">
+        <is>
+          <t>Bảng Giá Vàng SJC, 9999 Realtime &amp; Công Cụ Quy Đổi</t>
+        </is>
+      </c>
+      <c r="D17" s="187" t="inlineStr">
         <is>
           <t>/tai-chinh/gia-vang</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="98" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="99" t="inlineStr">
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="182" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="183" t="inlineStr">
         <is>
           <t>Công Cụ Tiện Ích Under /tai-chinh</t>
         </is>
       </c>
-      <c r="C8" s="100" t="inlineStr">
-        <is>
-          <t>Tính Lương Gross Sang Net 2026</t>
-        </is>
-      </c>
-      <c r="D8" s="101" t="inlineStr">
+      <c r="C18" s="178" t="inlineStr">
+        <is>
+          <t>Tính Lương Gross Sang Net &amp; Ngược Lại 2026</t>
+        </is>
+      </c>
+      <c r="D18" s="184" t="inlineStr">
         <is>
           <t>/tai-chinh/tinh-luong</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="98" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="99" t="inlineStr">
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="185" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="186" t="inlineStr">
         <is>
           <t>Công Cụ Tiện Ích Under /tai-chinh</t>
         </is>
       </c>
-      <c r="C9" s="100" t="inlineStr">
+      <c r="C19" s="172" t="inlineStr">
         <is>
           <t>Gửi Tiết Kiệm Online MoMo &amp; Lãi Suất Ưu Đãi Đối Tác</t>
         </is>
       </c>
-      <c r="D9" s="101" t="inlineStr">
+      <c r="D19" s="187" t="inlineStr">
         <is>
           <t>/tai-chinh/gui-tiet-kiem</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="98" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="99" t="inlineStr">
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="182" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="183" t="inlineStr">
         <is>
           <t>Công Cụ Tiện Ích Under /tai-chinh</t>
         </is>
       </c>
-      <c r="C10" s="100" t="inlineStr">
+      <c r="C20" s="178" t="inlineStr">
         <is>
           <t>Bảng Tra Cứu Lãi Suất 40 Ngân Hàng Toàn Cảnh Thị Trường</t>
         </is>
       </c>
-      <c r="D10" s="101" t="inlineStr">
+      <c r="D20" s="184" t="inlineStr">
         <is>
           <t>/tai-chinh/lai-suat</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="98" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="99" t="inlineStr">
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="185" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="186" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C21" s="172" t="inlineStr">
+        <is>
+          <t>Phân Bổ Lương 50/30/20 &amp; Hũ Tài Chính</t>
+        </is>
+      </c>
+      <c r="D21" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/phan-bo-luong</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="182" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="183" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C22" s="178" t="inlineStr">
+        <is>
+          <t>Bộ Giả Lập Tự Do Tài Chính &amp; Tích Sản FIRE</t>
+        </is>
+      </c>
+      <c r="D22" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/tu-do-tai-chinh</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="185" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="186" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C23" s="172" t="inlineStr">
+        <is>
+          <t>Dự Toán Lương Hưu &amp; Tuổi Nghỉ Hưu Luật Mới</t>
+        </is>
+      </c>
+      <c r="D23" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/luong-huu</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="182" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="183" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C24" s="178" t="inlineStr">
+        <is>
+          <t>Quản Lý Dòng Tiền Tự Do &amp; Quỹ Dự Phòng Khẩn Cấp</t>
+        </is>
+      </c>
+      <c r="D24" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/dong-tien</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="185" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="186" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C25" s="172" t="inlineStr">
+        <is>
+          <t>Cổng Tra Cứu &amp; Xác Thực Mã Số Thuế Cá Nhân</t>
+        </is>
+      </c>
+      <c r="D25" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ma-so-thue</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="182" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Chi Tiết (Programmatic Spoke)</t>
+        </is>
+      </c>
+      <c r="C26" s="178" t="inlineStr">
+        <is>
+          <t>Hệ Thống Dynamic Profile 30 Mã VN30 ([Mã Cổ Phiếu])</t>
+        </is>
+      </c>
+      <c r="D26" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/[ticker]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="185" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="186" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C27" s="172" t="inlineStr">
+        <is>
+          <t>Bảng Theo Dõi Lịch Cổ Tức Tiền Mặt Doanh Nghiệp</t>
+        </is>
+      </c>
+      <c r="D27" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/lich-co-tuc</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="182" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C28" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu FPT - CTCP FPT</t>
+        </is>
+      </c>
+      <c r="D28" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/fpt</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="185" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C29" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu VNM - CTCP Sữa Việt Nam (Vinamilk)</t>
+        </is>
+      </c>
+      <c r="D29" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/vnm</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="182" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C30" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu HPG - Tập Đoàn Hòa Phát</t>
+        </is>
+      </c>
+      <c r="D30" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/hpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="185" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C31" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu VCB - Ngân Hàng TMCP Ngoại Thương Việt Nam</t>
+        </is>
+      </c>
+      <c r="D31" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/vcb</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="182" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C32" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu MWG - CTCP Đầu Tư Thế Giới Di Động</t>
+        </is>
+      </c>
+      <c r="D32" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/mwg</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="185" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C33" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu TCB - Ngân Hàng TMCP Kỹ Thương Việt Nam</t>
+        </is>
+      </c>
+      <c r="D33" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/tcb</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="182" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C34" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu MBB - Ngân Hàng TMCP Quân Đội</t>
+        </is>
+      </c>
+      <c r="D34" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/mbb</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="185" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C35" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu ACB - Ngân Hàng TMCP Á Châu</t>
+        </is>
+      </c>
+      <c r="D35" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/acb</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="182" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C36" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu BID - Ngân Hàng TMCP Đầu Tư &amp; Phát Triển Việt Nam</t>
+        </is>
+      </c>
+      <c r="D36" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/bid</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="185" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C37" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu CTG - Ngân Hàng TMCP Công Thương Việt Nam</t>
+        </is>
+      </c>
+      <c r="D37" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/ctg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="182" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C38" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu MSN - CTCP Tập Đoàn Masan</t>
+        </is>
+      </c>
+      <c r="D38" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/msn</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="185" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C39" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu GAS - Tổng Công Ty Khí Việt Nam (PV GAS)</t>
+        </is>
+      </c>
+      <c r="D39" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/gas</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="182" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C40" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu VIC - Tập Đoàn Vingroup</t>
+        </is>
+      </c>
+      <c r="D40" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/vic</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="185" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C41" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu VHM - CTCP Vinhomes</t>
+        </is>
+      </c>
+      <c r="D41" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/vhm</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="182" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C42" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu VRE - CTCP Vincom Retail</t>
+        </is>
+      </c>
+      <c r="D42" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/vre</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="185" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C43" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu HDB - Ngân Hàng TMCP Phát Triển TP.HCM</t>
+        </is>
+      </c>
+      <c r="D43" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/hdb</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="182" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C44" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu STB - Ngân Hàng TMCP Sài Gòn Thương Tín</t>
+        </is>
+      </c>
+      <c r="D44" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/stb</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="185" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C45" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu TPB - Ngân Hàng TMCP Tiên Phong</t>
+        </is>
+      </c>
+      <c r="D45" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/tpb</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="182" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C46" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu VPB - Ngân Hàng TMCP Việt Nam Thịnh Vượng</t>
+        </is>
+      </c>
+      <c r="D46" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/vpb</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="185" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C47" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu VIB - Ngân Hàng TMCP Quốc Tế Việt Nam</t>
+        </is>
+      </c>
+      <c r="D47" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/vib</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="182" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C48" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu SHB - Ngân Hàng TMCP Sài Gòn - Hà Nội</t>
+        </is>
+      </c>
+      <c r="D48" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/shb</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="185" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C49" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu SSB - Ngân Hàng TMCP Đông Nam Á (SeABank)</t>
+        </is>
+      </c>
+      <c r="D49" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/ssb</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="182" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C50" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu SSI - CTCP Chứng Khoán SSI</t>
+        </is>
+      </c>
+      <c r="D50" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/ssi</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="185" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C51" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu PLX - Tập Đoàn Xăng Dầu Việt Nam (Petrolimex)</t>
+        </is>
+      </c>
+      <c r="D51" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/plx</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="182" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C52" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu POW - Tổng Công Ty Điện Lực Dầu Khí Việt Nam</t>
+        </is>
+      </c>
+      <c r="D52" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/pow</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="185" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C53" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu SAB - Tổng CTCP Bia - Rượu - Nước Giải Khát Sài Gòn</t>
+        </is>
+      </c>
+      <c r="D53" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/sab</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="182" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C54" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu BVH - Tập Đoàn Bảo Việt</t>
+        </is>
+      </c>
+      <c r="D54" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/bvh</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="185" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C55" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu BCM - Tổng Công Ty Đầu Tư &amp; Phát Triển Công Nghiệp</t>
+        </is>
+      </c>
+      <c r="D55" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/bcm</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="182" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C56" s="178" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu GVR - Tập Đoàn Công Nghiệp Cao Su Việt Nam</t>
+        </is>
+      </c>
+      <c r="D56" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/gvr</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="185" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cổ Phiếu (Programmatic VN30)</t>
+        </is>
+      </c>
+      <c r="C57" s="172" t="inlineStr">
+        <is>
+          <t>Cổ Phiếu VJC - CTCP Hàng Không Vietjet</t>
+        </is>
+      </c>
+      <c r="D57" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-khoan/vjc</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="182" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Chi Tiết (Programmatic Spoke)</t>
+        </is>
+      </c>
+      <c r="C58" s="178" t="inlineStr">
+        <is>
+          <t>Hệ Thống Trang Chi Tiết 30 Quỹ Mở Đối Tác CVS ([Tên Quỹ])</t>
+        </is>
+      </c>
+      <c r="D58" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/[fund-slug]</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="185" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" s="186" t="inlineStr">
+        <is>
+          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
+        </is>
+      </c>
+      <c r="C59" s="172" t="inlineStr">
+        <is>
+          <t>Máy Tính Giả Lập Tích Sản Định Kỳ SIP Quỹ Mở Từ 10.000đ</t>
+        </is>
+      </c>
+      <c r="D59" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/tich-san-sip</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="182" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Quỹ Mở (Programmatic CCQ)</t>
+        </is>
+      </c>
+      <c r="C60" s="178" t="inlineStr">
+        <is>
+          <t>Quỹ Đầu Tư Doanh Nghiệp Hàng Đầu Dragon Capital (DCDS)</t>
+        </is>
+      </c>
+      <c r="D60" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/dcds</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="185" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Quỹ Mở (Programmatic CCQ)</t>
+        </is>
+      </c>
+      <c r="C61" s="172" t="inlineStr">
+        <is>
+          <t>Quỹ Đầu Tư Cổ Phiếu Tiếp Cận Thị Trường VinaCapital (VESAF)</t>
+        </is>
+      </c>
+      <c r="D61" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/vesaf</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="182" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Quỹ Mở (Programmatic CCQ)</t>
+        </is>
+      </c>
+      <c r="C62" s="178" t="inlineStr">
+        <is>
+          <t>Quỹ Đầu Tư Cổ Phiếu Hưng Thịnh VinaCapital (VEOF)</t>
+        </is>
+      </c>
+      <c r="D62" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/veof</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="185" t="n">
+        <v>60</v>
+      </c>
+      <c r="B63" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Quỹ Mở (Programmatic CCQ)</t>
+        </is>
+      </c>
+      <c r="C63" s="172" t="inlineStr">
+        <is>
+          <t>Quỹ Đầu Tư Cổ Phiếu Tăng Trưởng VCBF (VCBF-MGF)</t>
+        </is>
+      </c>
+      <c r="D63" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/vcbf-mgf</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="182" t="n">
+        <v>61</v>
+      </c>
+      <c r="B64" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Quỹ Mở (Programmatic CCQ)</t>
+        </is>
+      </c>
+      <c r="C64" s="178" t="inlineStr">
+        <is>
+          <t>Quỹ Đầu Tư Cổ Phiếu Hàng Đầu VCBF (VCBF-BCF)</t>
+        </is>
+      </c>
+      <c r="D64" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/vcbf-bcf</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="185" t="n">
+        <v>62</v>
+      </c>
+      <c r="B65" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Quỹ Mở (Programmatic CCQ)</t>
+        </is>
+      </c>
+      <c r="C65" s="172" t="inlineStr">
+        <is>
+          <t>Quỹ Đầu Tư Lợi Thế Cạnh Tranh Bền Vững SSI (SSI-SCA)</t>
+        </is>
+      </c>
+      <c r="D65" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/ssi-sca</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="182" t="n">
+        <v>63</v>
+      </c>
+      <c r="B66" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Quỹ Mở (Programmatic CCQ)</t>
+        </is>
+      </c>
+      <c r="C66" s="178" t="inlineStr">
+        <is>
+          <t>Quỹ Đầu Tư Cổ Phiếu Triển Vọng Bảo Việt (BVBF)</t>
+        </is>
+      </c>
+      <c r="D66" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/bvbf</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="185" t="n">
+        <v>64</v>
+      </c>
+      <c r="B67" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Quỹ Mở (Programmatic CCQ)</t>
+        </is>
+      </c>
+      <c r="C67" s="172" t="inlineStr">
+        <is>
+          <t>Quỹ Đầu Tư Chứng Khoán Năng Động Dragon Capital (DCBC)</t>
+        </is>
+      </c>
+      <c r="D67" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/dcbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="182" t="n">
+        <v>65</v>
+      </c>
+      <c r="B68" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Quỹ Mở (Programmatic CCQ)</t>
+        </is>
+      </c>
+      <c r="C68" s="178" t="inlineStr">
+        <is>
+          <t>Quỹ Đầu Tư Cổ Phiếu Cổ Tức VinaCapital (VDEF)</t>
+        </is>
+      </c>
+      <c r="D68" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/vdef</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="185" t="n">
+        <v>66</v>
+      </c>
+      <c r="B69" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Quỹ Mở (Programmatic CCQ)</t>
+        </is>
+      </c>
+      <c r="C69" s="172" t="inlineStr">
+        <is>
+          <t>Quỹ Đầu Tư Cổ Phiếu Kinh Tế Hiện Đại VinaCapital (VMEEF)</t>
+        </is>
+      </c>
+      <c r="D69" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/chung-chi-quy/vmeef</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="182" t="n">
+        <v>67</v>
+      </c>
+      <c r="B70" s="183" t="inlineStr">
         <is>
           <t>Cổng Danh Mục Under /tai-chinh</t>
         </is>
       </c>
-      <c r="C11" s="100" t="inlineStr">
+      <c r="C70" s="178" t="inlineStr">
         <is>
           <t>Cổng Tỷ Giá Ngoại Tệ 20+ Ngân Hàng</t>
         </is>
       </c>
-      <c r="D11" s="101" t="inlineStr">
+      <c r="D70" s="184" t="inlineStr">
         <is>
           <t>/tai-chinh/ty-gia</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="98" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="99" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="185" t="n">
+        <v>68</v>
+      </c>
+      <c r="B71" s="186" t="inlineStr">
         <is>
           <t>Trang Con Cặp Tiền (Programmatic Subpage)</t>
         </is>
       </c>
-      <c r="C12" s="100" t="inlineStr">
+      <c r="C71" s="172" t="inlineStr">
         <is>
           <t>Hệ Thống Quy Đổi Ngoại Tệ Theo Cặp Tiền ([Đồng Tiền]/VND)</t>
         </is>
       </c>
-      <c r="D12" s="101" t="inlineStr">
+      <c r="D71" s="187" t="inlineStr">
         <is>
           <t>/tai-chinh/ty-gia/[pair-slug]</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="98" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="99" t="inlineStr">
-        <is>
-          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
-        </is>
-      </c>
-      <c r="C13" s="100" t="inlineStr">
-        <is>
-          <t>Phân Bổ Lương 50/30/20 &amp; Hũ Tài Chính</t>
-        </is>
-      </c>
-      <c r="D13" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/phan-bo-luong</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="98" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="99" t="inlineStr">
-        <is>
-          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
-        </is>
-      </c>
-      <c r="C14" s="100" t="inlineStr">
-        <is>
-          <t>Bộ Giả Lập Tự Do Tài Chính &amp; Tích Sản FIRE</t>
-        </is>
-      </c>
-      <c r="D14" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/tu-do-tai-chinh</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="98" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="99" t="inlineStr">
-        <is>
-          <t>Công Cụ Tiện Ích Under /tai-chinh</t>
-        </is>
-      </c>
-      <c r="C15" s="100" t="inlineStr">
-        <is>
-          <t>Dự Toán Lương Hưu &amp; Tuổi Nghỉ Hưu Mới Nhất</t>
-        </is>
-      </c>
-      <c r="D15" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/luong-huu</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="98" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="99" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="182" t="n">
+        <v>69</v>
+      </c>
+      <c r="B72" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cặp Tiền (Programmatic)</t>
+        </is>
+      </c>
+      <c r="C72" s="178" t="inlineStr">
+        <is>
+          <t>Tỷ Giá USD/VND Hôm Nay</t>
+        </is>
+      </c>
+      <c r="D72" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ty-gia/usd-vnd</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="185" t="n">
+        <v>70</v>
+      </c>
+      <c r="B73" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cặp Tiền (Programmatic)</t>
+        </is>
+      </c>
+      <c r="C73" s="172" t="inlineStr">
+        <is>
+          <t>Tỷ Giá EUR/VND Hôm Nay</t>
+        </is>
+      </c>
+      <c r="D73" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ty-gia/eur-vnd</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="182" t="n">
+        <v>71</v>
+      </c>
+      <c r="B74" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cặp Tiền (Programmatic)</t>
+        </is>
+      </c>
+      <c r="C74" s="178" t="inlineStr">
+        <is>
+          <t>Tỷ Giá Yên Nhật JPY/VND Hôm Nay</t>
+        </is>
+      </c>
+      <c r="D74" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ty-gia/jpy-vnd</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="185" t="n">
+        <v>72</v>
+      </c>
+      <c r="B75" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cặp Tiền (Programmatic)</t>
+        </is>
+      </c>
+      <c r="C75" s="172" t="inlineStr">
+        <is>
+          <t>Tỷ Giá Won Hàn KRW/VND Hôm Nay</t>
+        </is>
+      </c>
+      <c r="D75" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ty-gia/krw-vnd</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="182" t="n">
+        <v>73</v>
+      </c>
+      <c r="B76" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cặp Tiền (Programmatic)</t>
+        </is>
+      </c>
+      <c r="C76" s="178" t="inlineStr">
+        <is>
+          <t>Tỷ Giá Nhân Dân Tệ CNY/VND Hôm Nay</t>
+        </is>
+      </c>
+      <c r="D76" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ty-gia/cny-vnd</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="185" t="n">
+        <v>74</v>
+      </c>
+      <c r="B77" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cặp Tiền (Programmatic)</t>
+        </is>
+      </c>
+      <c r="C77" s="172" t="inlineStr">
+        <is>
+          <t>Tỷ Giá Bảng Anh GBP/VND Hôm Nay</t>
+        </is>
+      </c>
+      <c r="D77" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ty-gia/gbp-vnd</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="182" t="n">
+        <v>75</v>
+      </c>
+      <c r="B78" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Cặp Tiền (Programmatic)</t>
+        </is>
+      </c>
+      <c r="C78" s="178" t="inlineStr">
+        <is>
+          <t>Tỷ Giá Đô Úc AUD/VND Hôm Nay</t>
+        </is>
+      </c>
+      <c r="D78" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ty-gia/aud-vnd</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="185" t="n">
+        <v>76</v>
+      </c>
+      <c r="B79" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Cặp Tiền (Programmatic)</t>
+        </is>
+      </c>
+      <c r="C79" s="172" t="inlineStr">
+        <is>
+          <t>Tỷ Giá Đô Singapore SGD/VND Hôm Nay</t>
+        </is>
+      </c>
+      <c r="D79" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ty-gia/sgd-vnd</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="182" t="n">
+        <v>77</v>
+      </c>
+      <c r="B80" s="183" t="inlineStr">
         <is>
           <t>Cổng Danh Mục Master</t>
         </is>
       </c>
-      <c r="C16" s="100" t="inlineStr">
+      <c r="C80" s="178" t="inlineStr">
         <is>
           <t>Danh Bạ 34 Ngân Hàng Việt Nam (Lãi Suất &amp; Hotline)</t>
         </is>
       </c>
-      <c r="D16" s="101" t="inlineStr">
+      <c r="D80" s="184" t="inlineStr">
         <is>
           <t>/tai-chinh/ngan-hang</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="98" t="n">
-        <v>14</v>
-      </c>
-      <c r="B17" s="99" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="185" t="n">
+        <v>78</v>
+      </c>
+      <c r="B81" s="186" t="inlineStr">
         <is>
           <t>Trang Con Chi Tiết (Programmatic Spoke)</t>
         </is>
       </c>
-      <c r="C17" s="100" t="inlineStr">
+      <c r="C81" s="172" t="inlineStr">
         <is>
           <t>Hệ Thống Trang Chi Tiết 34 Ngân Hàng Đối Tác ([Tên Ngân Hàng])</t>
         </is>
       </c>
-      <c r="D17" s="101" t="inlineStr">
+      <c r="D81" s="187" t="inlineStr">
         <is>
           <t>/tai-chinh/ngan-hang/[bank-slug]</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="98" t="n">
-        <v>15</v>
-      </c>
-      <c r="B18" s="99" t="inlineStr">
-        <is>
-          <t>Chuyên Trang Độc Lập (Vertical Hub)</t>
-        </is>
-      </c>
-      <c r="C18" s="100" t="inlineStr">
-        <is>
-          <t>Bảng Giá Tra Cứu Chỉ Số Chứng Khoán (VN-Index, HNX)</t>
-        </is>
-      </c>
-      <c r="D18" s="101" t="inlineStr">
-        <is>
-          <t>/chung-khoan</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="98" t="n">
-        <v>16</v>
-      </c>
-      <c r="B19" s="99" t="inlineStr">
-        <is>
-          <t>Chuyên Trang Under /tai-chinh</t>
-        </is>
-      </c>
-      <c r="C19" s="100" t="inlineStr">
-        <is>
-          <t>Bảng Tra Cứu Giá NAV &amp; Tích Sản Quỹ Mở</t>
-        </is>
-      </c>
-      <c r="D19" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/chung-chi-quy</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="98" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="99" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="182" t="n">
+        <v>79</v>
+      </c>
+      <c r="B82" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C82" s="178" t="inlineStr">
+        <is>
+          <t>VietinBank - Ngân Hàng TMCP Công Thương Việt Nam</t>
+        </is>
+      </c>
+      <c r="D82" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/vietinbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="185" t="n">
+        <v>80</v>
+      </c>
+      <c r="B83" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C83" s="172" t="inlineStr">
+        <is>
+          <t>Vietcombank - Ngân Hàng TMCP Ngoại Thương Việt Nam</t>
+        </is>
+      </c>
+      <c r="D83" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/vietcombank</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="182" t="n">
+        <v>81</v>
+      </c>
+      <c r="B84" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C84" s="178" t="inlineStr">
+        <is>
+          <t>Techcombank - Ngân Hàng TMCP Kỹ Thương Việt Nam</t>
+        </is>
+      </c>
+      <c r="D84" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/techcombank</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="185" t="n">
+        <v>82</v>
+      </c>
+      <c r="B85" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C85" s="172" t="inlineStr">
+        <is>
+          <t>Nam A Bank - Ngân Hàng TMCP Nam Á</t>
+        </is>
+      </c>
+      <c r="D85" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/nam-a-bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="182" t="n">
+        <v>83</v>
+      </c>
+      <c r="B86" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C86" s="178" t="inlineStr">
+        <is>
+          <t>VPBank - Ngân Hàng TMCP Việt Nam Thịnh Vượng</t>
+        </is>
+      </c>
+      <c r="D86" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/vpbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="185" t="n">
+        <v>84</v>
+      </c>
+      <c r="B87" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C87" s="172" t="inlineStr">
+        <is>
+          <t>Agribank - Ngân Hàng Nông Nghiệp &amp; PTNT Việt Nam</t>
+        </is>
+      </c>
+      <c r="D87" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/agribank</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="182" t="n">
+        <v>85</v>
+      </c>
+      <c r="B88" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C88" s="178" t="inlineStr">
+        <is>
+          <t>MBBank - Ngân Hàng TMCP Quân Đội</t>
+        </is>
+      </c>
+      <c r="D88" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/mbbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="185" t="n">
+        <v>86</v>
+      </c>
+      <c r="B89" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C89" s="172" t="inlineStr">
+        <is>
+          <t>VRB - Ngân Hàng Liên Doanh Việt - Nga</t>
+        </is>
+      </c>
+      <c r="D89" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/vrb</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="182" t="n">
+        <v>87</v>
+      </c>
+      <c r="B90" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C90" s="178" t="inlineStr">
+        <is>
+          <t>ACB - Ngân Hàng TMCP Á Châu</t>
+        </is>
+      </c>
+      <c r="D90" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/acb</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="185" t="n">
+        <v>88</v>
+      </c>
+      <c r="B91" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C91" s="172" t="inlineStr">
+        <is>
+          <t>BIDV - Ngân Hàng TMCP Đầu Tư &amp; Phát Triển Việt Nam</t>
+        </is>
+      </c>
+      <c r="D91" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/bidv</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="182" t="n">
+        <v>89</v>
+      </c>
+      <c r="B92" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C92" s="178" t="inlineStr">
+        <is>
+          <t>MSB - Ngân Hàng TMCP Hàng Hải Việt Nam</t>
+        </is>
+      </c>
+      <c r="D92" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/msb</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="185" t="n">
+        <v>90</v>
+      </c>
+      <c r="B93" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C93" s="172" t="inlineStr">
+        <is>
+          <t>TPBank - Ngân Hàng TMCP Tiên Phong</t>
+        </is>
+      </c>
+      <c r="D93" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/tpbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="182" t="n">
+        <v>91</v>
+      </c>
+      <c r="B94" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C94" s="178" t="inlineStr">
+        <is>
+          <t>SCB - Ngân Hàng TMCP Sài Gòn</t>
+        </is>
+      </c>
+      <c r="D94" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/scb</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="185" t="n">
+        <v>92</v>
+      </c>
+      <c r="B95" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C95" s="172" t="inlineStr">
+        <is>
+          <t>SHB - Ngân Hàng TMCP Sài Gòn - Hà Nội</t>
+        </is>
+      </c>
+      <c r="D95" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/shb</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="182" t="n">
+        <v>93</v>
+      </c>
+      <c r="B96" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C96" s="178" t="inlineStr">
+        <is>
+          <t>Sacombank - Ngân Hàng TMCP Sài Gòn Thương Tín</t>
+        </is>
+      </c>
+      <c r="D96" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/sacombank</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="185" t="n">
+        <v>94</v>
+      </c>
+      <c r="B97" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C97" s="172" t="inlineStr">
+        <is>
+          <t>ABBank - Ngân Hàng TMCP An Bình</t>
+        </is>
+      </c>
+      <c r="D97" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/abbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="182" t="n">
+        <v>95</v>
+      </c>
+      <c r="B98" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C98" s="178" t="inlineStr">
+        <is>
+          <t>OCB - Ngân Hàng TMCP Phương Đông</t>
+        </is>
+      </c>
+      <c r="D98" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/ocb</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="185" t="n">
+        <v>96</v>
+      </c>
+      <c r="B99" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C99" s="172" t="inlineStr">
+        <is>
+          <t>Shinhan Bank - Ngân Hàng TNHH MTV Shinhan Việt Nam</t>
+        </is>
+      </c>
+      <c r="D99" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/shinhan-bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="182" t="n">
+        <v>97</v>
+      </c>
+      <c r="B100" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C100" s="178" t="inlineStr">
+        <is>
+          <t>NCB - Ngân Hàng TMCP Quốc Dân</t>
+        </is>
+      </c>
+      <c r="D100" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/ncb</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="185" t="n">
+        <v>98</v>
+      </c>
+      <c r="B101" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C101" s="172" t="inlineStr">
+        <is>
+          <t>Bản Việt (BVBank) - Ngân Hàng TMCP Bản Việt</t>
+        </is>
+      </c>
+      <c r="D101" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/bvbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="182" t="n">
+        <v>99</v>
+      </c>
+      <c r="B102" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C102" s="178" t="inlineStr">
+        <is>
+          <t>SeABank - Ngân Hàng TMCP Đông Nam Á</t>
+        </is>
+      </c>
+      <c r="D102" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/seabank</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="185" t="n">
+        <v>100</v>
+      </c>
+      <c r="B103" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C103" s="172" t="inlineStr">
+        <is>
+          <t>Eximbank - Ngân Hàng TMCP Xuất Nhập Khẩu Việt Nam</t>
+        </is>
+      </c>
+      <c r="D103" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/eximbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="182" t="n">
+        <v>101</v>
+      </c>
+      <c r="B104" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C104" s="178" t="inlineStr">
+        <is>
+          <t>VIB - Ngân Hàng TMCP Quốc Tế Việt Nam</t>
+        </is>
+      </c>
+      <c r="D104" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/vib</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="185" t="n">
+        <v>102</v>
+      </c>
+      <c r="B105" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C105" s="172" t="inlineStr">
+        <is>
+          <t>HDBank - Ngân Hàng TMCP Phát Triển TP.HCM</t>
+        </is>
+      </c>
+      <c r="D105" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/hdbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="182" t="n">
+        <v>103</v>
+      </c>
+      <c r="B106" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C106" s="178" t="inlineStr">
+        <is>
+          <t>VietBank - Ngân Hàng TMCP Việt Nam Thương Tín</t>
+        </is>
+      </c>
+      <c r="D106" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/vietbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="185" t="n">
+        <v>104</v>
+      </c>
+      <c r="B107" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C107" s="172" t="inlineStr">
+        <is>
+          <t>PVcomBank - Ngân Hàng TMCP Đại Chúng Việt Nam</t>
+        </is>
+      </c>
+      <c r="D107" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/pvcombank</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="182" t="n">
+        <v>105</v>
+      </c>
+      <c r="B108" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C108" s="178" t="inlineStr">
+        <is>
+          <t>DongA Bank - Ngân Hàng TMCP Đông Á</t>
+        </is>
+      </c>
+      <c r="D108" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/donga-bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="185" t="n">
+        <v>106</v>
+      </c>
+      <c r="B109" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C109" s="172" t="inlineStr">
+        <is>
+          <t>Bac A Bank - Ngân Hàng TMCP Bắc Á</t>
+        </is>
+      </c>
+      <c r="D109" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/bac-a-bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="182" t="n">
+        <v>107</v>
+      </c>
+      <c r="B110" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C110" s="178" t="inlineStr">
+        <is>
+          <t>LPBank - Ngân Hàng TMCP Lộc Phát Việt Nam</t>
+        </is>
+      </c>
+      <c r="D110" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/lpbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="185" t="n">
+        <v>108</v>
+      </c>
+      <c r="B111" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C111" s="172" t="inlineStr">
+        <is>
+          <t>KienlongBank - Ngân Hàng TMCP Kiên Long</t>
+        </is>
+      </c>
+      <c r="D111" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/kienlongbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="182" t="n">
+        <v>109</v>
+      </c>
+      <c r="B112" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C112" s="178" t="inlineStr">
+        <is>
+          <t>BaoViet Bank - Ngân Hàng TMCP Bảo Việt</t>
+        </is>
+      </c>
+      <c r="D112" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/baovietbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="185" t="n">
+        <v>110</v>
+      </c>
+      <c r="B113" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C113" s="172" t="inlineStr">
+        <is>
+          <t>Indovina Bank - Ngân Hàng TNHH Indovina (IVB)</t>
+        </is>
+      </c>
+      <c r="D113" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/indovina-bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="182" t="n">
+        <v>111</v>
+      </c>
+      <c r="B114" s="183" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C114" s="178" t="inlineStr">
+        <is>
+          <t>OceanBank - Ngân Hàng Thương Mại TNHH MTV Đại Dương</t>
+        </is>
+      </c>
+      <c r="D114" s="184" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/oceanbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="185" t="n">
+        <v>112</v>
+      </c>
+      <c r="B115" s="186" t="inlineStr">
+        <is>
+          <t>Trang Con Ngân Hàng (Programmatic Bank)</t>
+        </is>
+      </c>
+      <c r="C115" s="172" t="inlineStr">
+        <is>
+          <t>Saigonbank - Ngân Hàng TMCP Sài Gòn Công Thương</t>
+        </is>
+      </c>
+      <c r="D115" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/ngan-hang/saigonbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="182" t="n">
+        <v>113</v>
+      </c>
+      <c r="B116" s="183" t="inlineStr">
         <is>
           <t>Trang Danh Mục Blog (Blog Listing)</t>
         </is>
       </c>
-      <c r="C20" s="100" t="inlineStr">
-        <is>
-          <t>Cẩm Nang Tài Chính Cá Nhân &amp; Đầu Tư</t>
-        </is>
-      </c>
-      <c r="D20" s="101" t="inlineStr">
+      <c r="C116" s="178" t="inlineStr">
+        <is>
+          <t>Cẩm Nang Tài Chính Cá Nhân &amp; Đầu Tư MoMo</t>
+        </is>
+      </c>
+      <c r="D116" s="184" t="inlineStr">
         <is>
           <t>/tai-chinh/blog</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="98" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="99" t="inlineStr">
-        <is>
-          <t>Kho 50 Bài Viết Chi Tiết (Blog Details)</t>
-        </is>
-      </c>
-      <c r="C21" s="100" t="inlineStr">
-        <is>
-          <t>Kho 100 Bài Viết Chi Tiết (Blog Details)</t>
-        </is>
-      </c>
-      <c r="D21" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/blog/[slug] (100 bài: 50 T9 + 50 T10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="98" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="99" t="inlineStr">
-        <is>
-          <t>Trang Con Cặp Tiền (Programmatic)</t>
-        </is>
-      </c>
-      <c r="C22" s="100" t="inlineStr">
-        <is>
-          <t>Tỷ Giá USD/VND Hôm Nay</t>
-        </is>
-      </c>
-      <c r="D22" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/ty-gia/usd-vnd</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="98" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" s="99" t="inlineStr">
-        <is>
-          <t>Trang Con Cặp Tiền (Programmatic)</t>
-        </is>
-      </c>
-      <c r="C23" s="100" t="inlineStr">
-        <is>
-          <t>Tỷ Giá EUR/VND Hôm Nay</t>
-        </is>
-      </c>
-      <c r="D23" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/ty-gia/eur-vnd</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="98" t="n">
-        <v>21</v>
-      </c>
-      <c r="B24" s="99" t="inlineStr">
-        <is>
-          <t>Trang Con Cặp Tiền (Programmatic)</t>
-        </is>
-      </c>
-      <c r="C24" s="100" t="inlineStr">
-        <is>
-          <t>Tỷ Giá Yên Nhật JPY/VND Hôm Nay</t>
-        </is>
-      </c>
-      <c r="D24" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/ty-gia/jpy-vnd</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="98" t="n">
-        <v>22</v>
-      </c>
-      <c r="B25" s="99" t="inlineStr">
-        <is>
-          <t>Trang Con Cặp Tiền (Programmatic)</t>
-        </is>
-      </c>
-      <c r="C25" s="100" t="inlineStr">
-        <is>
-          <t>Tỷ Giá Won Hàn KRW/VND Hôm Nay</t>
-        </is>
-      </c>
-      <c r="D25" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/ty-gia/krw-vnd</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="A26" s="98" t="n">
-        <v>23</v>
-      </c>
-      <c r="B26" s="99" t="inlineStr">
-        <is>
-          <t>Trang Con Cặp Tiền (Programmatic)</t>
-        </is>
-      </c>
-      <c r="C26" s="100" t="inlineStr">
-        <is>
-          <t>Tỷ Giá Nhân Dân Tệ CNY/VND Hôm Nay</t>
-        </is>
-      </c>
-      <c r="D26" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/ty-gia/cny-vnd</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="26" customHeight="1">
-      <c r="A27" s="98" t="n">
-        <v>24</v>
-      </c>
-      <c r="B27" s="99" t="inlineStr">
-        <is>
-          <t>Trang Con Cặp Tiền (Programmatic)</t>
-        </is>
-      </c>
-      <c r="C27" s="100" t="inlineStr">
-        <is>
-          <t>Tỷ Giá Bảng Anh GBP/VND Hôm Nay</t>
-        </is>
-      </c>
-      <c r="D27" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/ty-gia/gbp-vnd</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="98" t="n">
-        <v>25</v>
-      </c>
-      <c r="B28" s="99" t="inlineStr">
-        <is>
-          <t>Trang Con Cặp Tiền (Programmatic)</t>
-        </is>
-      </c>
-      <c r="C28" s="100" t="inlineStr">
-        <is>
-          <t>Tỷ Giá Đô Úc AUD/VND Hôm Nay</t>
-        </is>
-      </c>
-      <c r="D28" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/ty-gia/aud-vnd</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="98" t="n">
-        <v>26</v>
-      </c>
-      <c r="B29" s="99" t="inlineStr">
-        <is>
-          <t>Trang Con Cặp Tiền (Programmatic)</t>
-        </is>
-      </c>
-      <c r="C29" s="100" t="inlineStr">
-        <is>
-          <t>Tỷ Giá Đô Singapore SGD/VND Hôm Nay</t>
-        </is>
-      </c>
-      <c r="D29" s="101" t="inlineStr">
-        <is>
-          <t>/tai-chinh/ty-gia/sgd-vnd</t>
+    <row r="117">
+      <c r="A117" s="185" t="n">
+        <v>114</v>
+      </c>
+      <c r="B117" s="186" t="inlineStr">
+        <is>
+          <t>Kho Bài Viết Chi Tiết (Blog Details)</t>
+        </is>
+      </c>
+      <c r="C117" s="172" t="inlineStr">
+        <is>
+          <t>Kho 100 Bài Viết Chi Tiết Chuẩn SEO &amp; GEO (50 T9 + 50 T10)</t>
+        </is>
+      </c>
+      <c r="D117" s="187" t="inlineStr">
+        <is>
+          <t>/tai-chinh/blog/[slug]</t>
         </is>
       </c>
     </row>

</xml_diff>